<commit_message>
Tune GDIT workforce demo data generation
Co-Authored-By: Chase Dalton <chase.dalton@cognition.ai>
</commit_message>
<xml_diff>
--- a/gdit-workforce-demo/data/finance/fy_headcount_budget.xlsx
+++ b/gdit-workforce-demo/data/finance/fy_headcount_budget.xlsx
@@ -470,10 +470,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>336.35</v>
+        <v>393.57</v>
       </c>
       <c r="F2" t="n">
-        <v>48983677.53</v>
+        <v>55627998.98</v>
       </c>
     </row>
     <row r="3">
@@ -498,10 +498,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>312</v>
+        <v>410</v>
       </c>
       <c r="F3" t="n">
-        <v>44148688.69</v>
+        <v>57314975.11</v>
       </c>
     </row>
     <row r="4">
@@ -526,10 +526,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>299.6</v>
+        <v>422.62</v>
       </c>
       <c r="F4" t="n">
-        <v>43360561.34</v>
+        <v>59521264.59</v>
       </c>
     </row>
     <row r="5">
@@ -554,10 +554,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>334.33</v>
+        <v>436.51</v>
       </c>
       <c r="F5" t="n">
-        <v>46747375.2</v>
+        <v>62333830.41</v>
       </c>
     </row>
     <row r="6">
@@ -582,10 +582,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>297.38</v>
+        <v>457.66</v>
       </c>
       <c r="F6" t="n">
-        <v>42569361.16</v>
+        <v>64660473.56</v>
       </c>
     </row>
     <row r="7">
@@ -610,10 +610,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>205.36</v>
+        <v>249.01</v>
       </c>
       <c r="F7" t="n">
-        <v>28706322.43</v>
+        <v>35091727.29</v>
       </c>
     </row>
     <row r="8">
@@ -638,10 +638,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>177.42</v>
+        <v>255.04</v>
       </c>
       <c r="F8" t="n">
-        <v>25448192.49</v>
+        <v>36126290.57</v>
       </c>
     </row>
     <row r="9">
@@ -666,10 +666,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>204.64</v>
+        <v>287.3</v>
       </c>
       <c r="F9" t="n">
-        <v>28529255.56</v>
+        <v>40413394.98</v>
       </c>
     </row>
     <row r="10">
@@ -694,10 +694,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>175.3</v>
+        <v>262.95</v>
       </c>
       <c r="F10" t="n">
-        <v>24658311.93</v>
+        <v>37890786.63</v>
       </c>
     </row>
     <row r="11">
@@ -722,10 +722,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>170.63</v>
+        <v>264.88</v>
       </c>
       <c r="F11" t="n">
-        <v>23605561.39</v>
+        <v>37981545.76</v>
       </c>
     </row>
     <row r="12">
@@ -750,10 +750,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="F12" t="n">
-        <v>57985441.64</v>
+        <v>63792248.06</v>
       </c>
     </row>
     <row r="13">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>366.53</v>
+        <v>487.05</v>
       </c>
       <c r="F13" t="n">
-        <v>51897889.67</v>
+        <v>68472745.75</v>
       </c>
     </row>
     <row r="14">
@@ -806,10 +806,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>368.95</v>
+        <v>488.91</v>
       </c>
       <c r="F14" t="n">
-        <v>52985479.7</v>
+        <v>69092999.62</v>
       </c>
     </row>
     <row r="15">
@@ -834,10 +834,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>398.19</v>
+        <v>494.96</v>
       </c>
       <c r="F15" t="n">
-        <v>56010966.26</v>
+        <v>70226939.38</v>
       </c>
     </row>
     <row r="16">
@@ -862,10 +862,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>355.42</v>
+        <v>522.09</v>
       </c>
       <c r="F16" t="n">
-        <v>50617295.33</v>
+        <v>73912246.61</v>
       </c>
     </row>
     <row r="17">
@@ -890,10 +890,10 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>248.99</v>
+        <v>304.44</v>
       </c>
       <c r="F17" t="n">
-        <v>34836348.48</v>
+        <v>43290447.18</v>
       </c>
     </row>
     <row r="18">
@@ -918,10 +918,10 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>219.88</v>
+        <v>287.15</v>
       </c>
       <c r="F18" t="n">
-        <v>31290148.25</v>
+        <v>40283020.43</v>
       </c>
     </row>
     <row r="19">
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>251</v>
+        <v>331.33</v>
       </c>
       <c r="F19" t="n">
-        <v>35459703.79</v>
+        <v>46389640.68</v>
       </c>
     </row>
     <row r="20">
@@ -974,10 +974,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>205.36</v>
+        <v>296.63</v>
       </c>
       <c r="F20" t="n">
-        <v>28886451.58</v>
+        <v>42846572.26</v>
       </c>
     </row>
     <row r="21">
@@ -1002,10 +1002,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>212.7</v>
+        <v>320.56</v>
       </c>
       <c r="F21" t="n">
-        <v>29521113.32</v>
+        <v>45999099.81</v>
       </c>
     </row>
     <row r="22">
@@ -1030,10 +1030,10 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>448.21</v>
+        <v>536.85</v>
       </c>
       <c r="F22" t="n">
-        <v>64626024.57</v>
+        <v>76599210.31</v>
       </c>
     </row>
     <row r="23">
@@ -1058,10 +1058,10 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>415.67</v>
+        <v>549.6</v>
       </c>
       <c r="F23" t="n">
-        <v>58804215.15</v>
+        <v>77239188.72</v>
       </c>
     </row>
     <row r="24">
@@ -1086,10 +1086,10 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>413.65</v>
+        <v>592.37</v>
       </c>
       <c r="F24" t="n">
-        <v>59662456.28</v>
+        <v>83839755.43000001</v>
       </c>
     </row>
     <row r="25">
@@ -1114,10 +1114,10 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>463.86</v>
+        <v>600.4</v>
       </c>
       <c r="F25" t="n">
-        <v>65579267.3</v>
+        <v>85449164.59</v>
       </c>
     </row>
     <row r="26">
@@ -1142,10 +1142,10 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>418</v>
+        <v>617</v>
       </c>
       <c r="F26" t="n">
-        <v>59300884.94</v>
+        <v>87840102.83</v>
       </c>
     </row>
     <row r="27">
@@ -1170,10 +1170,10 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>287.15</v>
+        <v>366.47</v>
       </c>
       <c r="F27" t="n">
-        <v>40050169.04</v>
+        <v>51786570.41</v>
       </c>
     </row>
     <row r="28">
@@ -1198,10 +1198,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>273</v>
+        <v>349</v>
       </c>
       <c r="F28" t="n">
-        <v>38645083.52</v>
+        <v>48876160.4</v>
       </c>
     </row>
     <row r="29">
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>303</v>
+        <v>386</v>
       </c>
       <c r="F29" t="n">
-        <v>43008515.41</v>
+        <v>53957910.92</v>
       </c>
     </row>
     <row r="30">
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>248.99</v>
+        <v>363.91</v>
       </c>
       <c r="F30" t="n">
-        <v>34933631.28</v>
+        <v>52269502.95</v>
       </c>
     </row>
     <row r="31">
@@ -1282,10 +1282,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>242.97</v>
+        <v>370.48</v>
       </c>
       <c r="F31" t="n">
-        <v>33906659.35</v>
+        <v>53147880.87</v>
       </c>
     </row>
     <row r="32">
@@ -1310,10 +1310,10 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>498.02</v>
+        <v>579.37</v>
       </c>
       <c r="F32" t="n">
-        <v>71673465.23</v>
+        <v>82257774.55</v>
       </c>
     </row>
     <row r="33">
@@ -1338,10 +1338,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>485.89</v>
+        <v>617.9400000000001</v>
       </c>
       <c r="F33" t="n">
-        <v>69004258.38</v>
+        <v>86807604.45</v>
       </c>
     </row>
     <row r="34">
@@ -1366,10 +1366,10 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>464</v>
+        <v>646</v>
       </c>
       <c r="F34" t="n">
-        <v>67094797.41</v>
+        <v>91085645.68000001</v>
       </c>
     </row>
     <row r="35">
@@ -1394,10 +1394,10 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>515</v>
+        <v>654</v>
       </c>
       <c r="F35" t="n">
-        <v>73327825.31</v>
+        <v>92539487.38</v>
       </c>
     </row>
     <row r="36">
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>482.07</v>
+        <v>645.42</v>
       </c>
       <c r="F36" t="n">
-        <v>68268448.36</v>
+        <v>91902063.06999999</v>
       </c>
     </row>
     <row r="37">
@@ -1450,10 +1450,10 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="F37" t="n">
-        <v>45132447.46</v>
+        <v>54730504.3</v>
       </c>
     </row>
     <row r="38">
@@ -1478,10 +1478,10 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>324.7</v>
+        <v>391.43</v>
       </c>
       <c r="F38" t="n">
-        <v>45362515.88</v>
+        <v>54543549.62</v>
       </c>
     </row>
     <row r="39">
@@ -1506,10 +1506,10 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>341.63</v>
+        <v>415.34</v>
       </c>
       <c r="F39" t="n">
-        <v>48591427.48</v>
+        <v>58131340.64</v>
       </c>
     </row>
     <row r="40">
@@ -1534,10 +1534,10 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>291.16</v>
+        <v>398.59</v>
       </c>
       <c r="F40" t="n">
-        <v>40923859.92</v>
+        <v>56890360.92</v>
       </c>
     </row>
     <row r="41">
@@ -1562,10 +1562,10 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>273</v>
+        <v>409</v>
       </c>
       <c r="F41" t="n">
-        <v>38045282.08</v>
+        <v>58901466.55</v>
       </c>
     </row>
     <row r="42">
@@ -1590,10 +1590,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>566</v>
+        <v>679</v>
       </c>
       <c r="F42" t="n">
-        <v>80994151.02</v>
+        <v>96291201.8</v>
       </c>
     </row>
     <row r="43">
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>541.83</v>
+        <v>690.24</v>
       </c>
       <c r="F43" t="n">
-        <v>76887519.69</v>
+        <v>96894330</v>
       </c>
     </row>
     <row r="44">
@@ -1646,10 +1646,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>508.06</v>
+        <v>728.83</v>
       </c>
       <c r="F44" t="n">
-        <v>73403980.94</v>
+        <v>103040687.82</v>
       </c>
     </row>
     <row r="45">
@@ -1674,10 +1674,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>599.8</v>
+        <v>730.85</v>
       </c>
       <c r="F45" t="n">
-        <v>85373245.23</v>
+        <v>103704293.05</v>
       </c>
     </row>
     <row r="46">
@@ -1702,10 +1702,10 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>565.26</v>
+        <v>730.92</v>
       </c>
       <c r="F46" t="n">
-        <v>79543716.78</v>
+        <v>104140885.83</v>
       </c>
     </row>
     <row r="47">
@@ -1730,10 +1730,10 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>360.89</v>
+        <v>459.68</v>
       </c>
       <c r="F47" t="n">
-        <v>50388665.67</v>
+        <v>64846959.6</v>
       </c>
     </row>
     <row r="48">
@@ -1758,10 +1758,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>355.42</v>
+        <v>465.86</v>
       </c>
       <c r="F48" t="n">
-        <v>49750954.27</v>
+        <v>65210258.52</v>
       </c>
     </row>
     <row r="49">
@@ -1786,10 +1786,10 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>377.51</v>
+        <v>493.98</v>
       </c>
       <c r="F49" t="n">
-        <v>53799437.84</v>
+        <v>69883696.06999999</v>
       </c>
     </row>
     <row r="50">
@@ -1814,10 +1814,10 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>318.45</v>
+        <v>445.44</v>
       </c>
       <c r="F50" t="n">
-        <v>44887165.92</v>
+        <v>63872859.88</v>
       </c>
     </row>
     <row r="51">
@@ -1842,10 +1842,10 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>311.49</v>
+        <v>467.74</v>
       </c>
       <c r="F51" t="n">
-        <v>43623268.68</v>
+        <v>67367885.58</v>
       </c>
     </row>
     <row r="52">
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>614.54</v>
+        <v>733.0700000000001</v>
       </c>
       <c r="F52" t="n">
-        <v>87792373.48999999</v>
+        <v>104107584.23</v>
       </c>
     </row>
     <row r="53">
@@ -1898,10 +1898,10 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>602.1799999999999</v>
+        <v>742.0599999999999</v>
       </c>
       <c r="F53" t="n">
-        <v>85679328.87</v>
+        <v>104035098.98</v>
       </c>
     </row>
     <row r="54">
@@ -1926,10 +1926,10 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>567.27</v>
+        <v>775.1</v>
       </c>
       <c r="F54" t="n">
-        <v>81685435.40000001</v>
+        <v>109403223.34</v>
       </c>
     </row>
     <row r="55">
@@ -1954,10 +1954,10 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>650.6</v>
+        <v>780.12</v>
       </c>
       <c r="F55" t="n">
-        <v>92233980.43000001</v>
+        <v>110126551.47</v>
       </c>
     </row>
     <row r="56">
@@ -1982,10 +1982,10 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>622</v>
+        <v>768</v>
       </c>
       <c r="F56" t="n">
-        <v>87935672.31999999</v>
+        <v>109708544.74</v>
       </c>
     </row>
     <row r="57">
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>399.6</v>
+        <v>505.02</v>
       </c>
       <c r="F57" t="n">
-        <v>56033448.15</v>
+        <v>71351957.33</v>
       </c>
     </row>
     <row r="58">
@@ -2038,10 +2038,10 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>382</v>
+        <v>517</v>
       </c>
       <c r="F58" t="n">
-        <v>53883858.48</v>
+        <v>72463306.66</v>
       </c>
     </row>
     <row r="59">
@@ -2066,10 +2066,10 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>419</v>
+        <v>532</v>
       </c>
       <c r="F59" t="n">
-        <v>59762752.92</v>
+        <v>75202714.45999999</v>
       </c>
     </row>
     <row r="60">
@@ -2094,10 +2094,10 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>349.8</v>
+        <v>491.94</v>
       </c>
       <c r="F60" t="n">
-        <v>49315829.19</v>
+        <v>70289089.52</v>
       </c>
     </row>
     <row r="61">
@@ -2122,10 +2122,10 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>353.41</v>
+        <v>487.95</v>
       </c>
       <c r="F61" t="n">
-        <v>49701213.35</v>
+        <v>70022194.12</v>
       </c>
     </row>
     <row r="62">
@@ -2150,10 +2150,10 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>665.67</v>
+        <v>790.67</v>
       </c>
       <c r="F62" t="n">
-        <v>94907099.81999999</v>
+        <v>112736279.14</v>
       </c>
     </row>
     <row r="63">
@@ -2178,10 +2178,10 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>665.3200000000001</v>
+        <v>840.73</v>
       </c>
       <c r="F63" t="n">
-        <v>94911541.68000001</v>
+        <v>117641443.76</v>
       </c>
     </row>
     <row r="64">
@@ -2206,10 +2206,10 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>623</v>
+        <v>842</v>
       </c>
       <c r="F64" t="n">
-        <v>89622014.66</v>
+        <v>119091743.76</v>
       </c>
     </row>
     <row r="65">
@@ -2234,10 +2234,10 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>690</v>
+        <v>860</v>
       </c>
       <c r="F65" t="n">
-        <v>97838148.14</v>
+        <v>121525085.08</v>
       </c>
     </row>
     <row r="66">
@@ -2262,10 +2262,10 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>675.3</v>
+        <v>869.52</v>
       </c>
       <c r="F66" t="n">
-        <v>95505152.12</v>
+        <v>124229413.18</v>
       </c>
     </row>
     <row r="67">
@@ -2290,10 +2290,10 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>434</v>
+        <v>551</v>
       </c>
       <c r="F67" t="n">
-        <v>60820103.31</v>
+        <v>77940626.09999999</v>
       </c>
     </row>
     <row r="68">
@@ -2318,10 +2318,10 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>425.3</v>
+        <v>567.73</v>
       </c>
       <c r="F68" t="n">
-        <v>59656035.82</v>
+        <v>79793390.83</v>
       </c>
     </row>
     <row r="69">
@@ -2346,10 +2346,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>449.2</v>
+        <v>576.6900000000001</v>
       </c>
       <c r="F69" t="n">
-        <v>63786340.82</v>
+        <v>81523169.39</v>
       </c>
     </row>
     <row r="70">
@@ -2374,10 +2374,10 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>386.55</v>
+        <v>533.13</v>
       </c>
       <c r="F70" t="n">
-        <v>54504664.21</v>
+        <v>76294918.26000001</v>
       </c>
     </row>
     <row r="71">
@@ -2402,10 +2402,10 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>384</v>
+        <v>547</v>
       </c>
       <c r="F71" t="n">
-        <v>53966391.62</v>
+        <v>78320067.08</v>
       </c>
     </row>
     <row r="72">
@@ -2430,10 +2430,10 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>721.77</v>
+        <v>858.87</v>
       </c>
       <c r="F72" t="n">
-        <v>103154898.67</v>
+        <v>121980038.27</v>
       </c>
     </row>
     <row r="73">
@@ -2458,10 +2458,10 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>710.84</v>
+        <v>892.5700000000001</v>
       </c>
       <c r="F73" t="n">
-        <v>101599986.05</v>
+        <v>125168527.25</v>
       </c>
     </row>
     <row r="74">
@@ -2486,10 +2486,10 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>676.29</v>
+        <v>883.47</v>
       </c>
       <c r="F74" t="n">
-        <v>97184436.41</v>
+        <v>125029963.45</v>
       </c>
     </row>
     <row r="75">
@@ -2514,10 +2514,10 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>743.03</v>
+        <v>911.35</v>
       </c>
       <c r="F75" t="n">
-        <v>105331243.05</v>
+        <v>129066255.41</v>
       </c>
     </row>
     <row r="76">
@@ -2542,10 +2542,10 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>717.26</v>
+        <v>923.61</v>
       </c>
       <c r="F76" t="n">
-        <v>101636925.93</v>
+        <v>132121016.37</v>
       </c>
     </row>
     <row r="77">
@@ -2570,10 +2570,10 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>477.09</v>
+        <v>579.6799999999999</v>
       </c>
       <c r="F77" t="n">
-        <v>66703147.38</v>
+        <v>81825841.84999999</v>
       </c>
     </row>
     <row r="78">
@@ -2598,10 +2598,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>464.29</v>
+        <v>607.14</v>
       </c>
       <c r="F78" t="n">
-        <v>65112017.39</v>
+        <v>85232695.19</v>
       </c>
     </row>
     <row r="79">
@@ -2626,10 +2626,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>487.1</v>
+        <v>615.08</v>
       </c>
       <c r="F79" t="n">
-        <v>69304672.45</v>
+        <v>86608329.64</v>
       </c>
     </row>
     <row r="80">
@@ -2654,10 +2654,10 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>428</v>
+        <v>550</v>
       </c>
       <c r="F80" t="n">
-        <v>59982651.38</v>
+        <v>78383151.37</v>
       </c>
     </row>
     <row r="81">
@@ -2682,10 +2682,10 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>412.35</v>
+        <v>569.72</v>
       </c>
       <c r="F81" t="n">
-        <v>58154509.6</v>
+        <v>81151397.02</v>
       </c>
     </row>
     <row r="82">
@@ -2710,10 +2710,10 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>766.9299999999999</v>
+        <v>933.27</v>
       </c>
       <c r="F82" t="n">
-        <v>109147006.16</v>
+        <v>132330832.86</v>
       </c>
     </row>
     <row r="83">
@@ -2738,10 +2738,10 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>739.09</v>
+        <v>955.36</v>
       </c>
       <c r="F83" t="n">
-        <v>105588503.11</v>
+        <v>134272969.14</v>
       </c>
     </row>
     <row r="84">
@@ -2766,10 +2766,10 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>727.91</v>
+        <v>951.8099999999999</v>
       </c>
       <c r="F84" t="n">
-        <v>104391085.77</v>
+        <v>134530701.97</v>
       </c>
     </row>
     <row r="85">
@@ -2794,10 +2794,10 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>802.21</v>
+        <v>1008.03</v>
       </c>
       <c r="F85" t="n">
-        <v>114070775.99</v>
+        <v>143079097.64</v>
       </c>
     </row>
     <row r="86">
@@ -2822,10 +2822,10 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>779</v>
+        <v>1001</v>
       </c>
       <c r="F86" t="n">
-        <v>110212102.51</v>
+        <v>143088211.8</v>
       </c>
     </row>
     <row r="87">
@@ -2850,10 +2850,10 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>528.11</v>
+        <v>625.5</v>
       </c>
       <c r="F87" t="n">
-        <v>73854965.38</v>
+        <v>88234324.06</v>
       </c>
     </row>
     <row r="88">
@@ -2878,10 +2878,10 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>503</v>
+        <v>662</v>
       </c>
       <c r="F88" t="n">
-        <v>70346519.91</v>
+        <v>92899159.48</v>
       </c>
     </row>
     <row r="89">
@@ -2906,10 +2906,10 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>525</v>
+        <v>669</v>
       </c>
       <c r="F89" t="n">
-        <v>74613490.11</v>
+        <v>94062577.95999999</v>
       </c>
     </row>
     <row r="90">
@@ -2934,10 +2934,10 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>472.78</v>
+        <v>592.74</v>
       </c>
       <c r="F90" t="n">
-        <v>66739194.36</v>
+        <v>83991091.28</v>
       </c>
     </row>
     <row r="91">
@@ -2962,10 +2962,10 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>445.78</v>
+        <v>607.4299999999999</v>
       </c>
       <c r="F91" t="n">
-        <v>62792806.94</v>
+        <v>86756407.31999999</v>
       </c>
     </row>
     <row r="92">
@@ -2990,10 +2990,10 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>813.49</v>
+        <v>978.17</v>
       </c>
       <c r="F92" t="n">
-        <v>115640964.99</v>
+        <v>138800441.08</v>
       </c>
     </row>
     <row r="93">
@@ -3018,10 +3018,10 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>808.47</v>
+        <v>1015.12</v>
       </c>
       <c r="F93" t="n">
-        <v>115393624.96</v>
+        <v>142373739.26</v>
       </c>
     </row>
     <row r="94">
@@ -3046,10 +3046,10 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>780</v>
+        <v>1001</v>
       </c>
       <c r="F94" t="n">
-        <v>112001067.58</v>
+        <v>141449526.02</v>
       </c>
     </row>
     <row r="95">
@@ -3074,10 +3074,10 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>853</v>
+        <v>1053</v>
       </c>
       <c r="F95" t="n">
-        <v>121834826.3</v>
+        <v>149005565.42</v>
       </c>
     </row>
     <row r="96">
@@ -3102,10 +3102,10 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>827.6900000000001</v>
+        <v>1029.88</v>
       </c>
       <c r="F96" t="n">
-        <v>117059556.95</v>
+        <v>146977165.38</v>
       </c>
     </row>
     <row r="97">
@@ -3130,10 +3130,10 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>560</v>
+        <v>658</v>
       </c>
       <c r="F97" t="n">
-        <v>78187547.48</v>
+        <v>92884140.97</v>
       </c>
     </row>
     <row r="98">
@@ -3158,10 +3158,10 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>547.8099999999999</v>
+        <v>694.22</v>
       </c>
       <c r="F98" t="n">
-        <v>76867656.13</v>
+        <v>97348220.95999999</v>
       </c>
     </row>
     <row r="99">
@@ -3186,10 +3186,10 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>574.7</v>
+        <v>689.24</v>
       </c>
       <c r="F99" t="n">
-        <v>81904603.48</v>
+        <v>96833283.13</v>
       </c>
     </row>
     <row r="100">
@@ -3214,10 +3214,10 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>505.02</v>
+        <v>626.51</v>
       </c>
       <c r="F100" t="n">
-        <v>71621961.8</v>
+        <v>89472191.84</v>
       </c>
     </row>
     <row r="101">
@@ -3242,10 +3242,10 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>479</v>
+        <v>632</v>
       </c>
       <c r="F101" t="n">
-        <v>67925784.45999999</v>
+        <v>90122755.53</v>
       </c>
     </row>
     <row r="102">
@@ -3270,10 +3270,10 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>875</v>
+        <v>1042.34</v>
       </c>
       <c r="F102" t="n">
-        <v>124203002.53</v>
+        <v>148289810.34</v>
       </c>
     </row>
     <row r="103">
@@ -3298,10 +3298,10 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>865.46</v>
+        <v>1064.26</v>
       </c>
       <c r="F103" t="n">
-        <v>123275613.5</v>
+        <v>149868684.22</v>
       </c>
     </row>
     <row r="104">
@@ -3326,10 +3326,10 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>818.73</v>
+        <v>1087.65</v>
       </c>
       <c r="F104" t="n">
-        <v>117496729.57</v>
+        <v>153501822.09</v>
       </c>
     </row>
     <row r="105">
@@ -3354,10 +3354,10 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>913.35</v>
+        <v>1115.54</v>
       </c>
       <c r="F105" t="n">
-        <v>130646788.04</v>
+        <v>157338291.53</v>
       </c>
     </row>
     <row r="106">
@@ -3382,10 +3382,10 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>861.11</v>
+        <v>1110.12</v>
       </c>
       <c r="F106" t="n">
-        <v>121858885.37</v>
+        <v>158297682.96</v>
       </c>
     </row>
     <row r="107">
@@ -3410,10 +3410,10 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>594.62</v>
+        <v>687.25</v>
       </c>
       <c r="F107" t="n">
-        <v>83310965.8</v>
+        <v>97213999.81</v>
       </c>
     </row>
     <row r="108">
@@ -3438,10 +3438,10 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>581.35</v>
+        <v>734.13</v>
       </c>
       <c r="F108" t="n">
-        <v>81731143.43000001</v>
+        <v>103113400.21</v>
       </c>
     </row>
     <row r="109">
@@ -3466,10 +3466,10 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>611.11</v>
+        <v>730.16</v>
       </c>
       <c r="F109" t="n">
-        <v>87130244.84999999</v>
+        <v>102775970.44</v>
       </c>
     </row>
     <row r="110">
@@ -3494,10 +3494,10 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>530</v>
+        <v>652</v>
       </c>
       <c r="F110" t="n">
-        <v>75312483.91</v>
+        <v>92971761.91</v>
       </c>
     </row>
     <row r="111">
@@ -3522,10 +3522,10 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>503.98</v>
+        <v>664.34</v>
       </c>
       <c r="F111" t="n">
-        <v>71319640.12</v>
+        <v>94909661.64</v>
       </c>
     </row>
     <row r="112">
@@ -3550,10 +3550,10 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>901.61</v>
+        <v>1062.25</v>
       </c>
       <c r="F112" t="n">
-        <v>128102887.62</v>
+        <v>151133689.47</v>
       </c>
     </row>
     <row r="113">
@@ -3578,10 +3578,10 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>913</v>
+        <v>1091</v>
       </c>
       <c r="F113" t="n">
-        <v>129440899.09</v>
+        <v>153269447.59</v>
       </c>
     </row>
     <row r="114">
@@ -3606,10 +3606,10 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>856.15</v>
+        <v>1124.01</v>
       </c>
       <c r="F114" t="n">
-        <v>122762747.65</v>
+        <v>158499071.38</v>
       </c>
     </row>
     <row r="115">
@@ -3634,10 +3634,10 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>958.33</v>
+        <v>1154.76</v>
       </c>
       <c r="F115" t="n">
-        <v>137199124.87</v>
+        <v>162636828.87</v>
       </c>
     </row>
     <row r="116">
@@ -3662,10 +3662,10 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>918.35</v>
+        <v>1167.34</v>
       </c>
       <c r="F116" t="n">
-        <v>129911995.23</v>
+        <v>166862638.72</v>
       </c>
     </row>
     <row r="117">
@@ -3690,10 +3690,10 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>625</v>
+        <v>712.3</v>
       </c>
       <c r="F117" t="n">
-        <v>87705275.51000001</v>
+        <v>100663600.1</v>
       </c>
     </row>
     <row r="118">
@@ -3718,10 +3718,10 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>615.9299999999999</v>
+        <v>777.22</v>
       </c>
       <c r="F118" t="n">
-        <v>86697778.05</v>
+        <v>108687131.38</v>
       </c>
     </row>
     <row r="119">
@@ -3746,10 +3746,10 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>655.24</v>
+        <v>762.1</v>
       </c>
       <c r="F119" t="n">
-        <v>93276111.73999999</v>
+        <v>106986316.66</v>
       </c>
     </row>
     <row r="120">
@@ -3774,10 +3774,10 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>561.75</v>
+        <v>676.29</v>
       </c>
       <c r="F120" t="n">
-        <v>79927998.3</v>
+        <v>96570630.18000001</v>
       </c>
     </row>
     <row r="121">
@@ -3802,10 +3802,10 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>534.72</v>
+        <v>679.5599999999999</v>
       </c>
       <c r="F121" t="n">
-        <v>75840753.01000001</v>
+        <v>97006889.76000001</v>
       </c>
     </row>
     <row r="122">
@@ -3830,10 +3830,10 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>935.52</v>
+        <v>1095.24</v>
       </c>
       <c r="F122" t="n">
-        <v>132601071.6</v>
+        <v>155665695.28</v>
       </c>
     </row>
     <row r="123">
@@ -3858,10 +3858,10 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>964.72</v>
+        <v>1166.33</v>
       </c>
       <c r="F123" t="n">
-        <v>136636767.01</v>
+        <v>163849116.21</v>
       </c>
     </row>
     <row r="124">
@@ -3886,10 +3886,10 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>904</v>
+        <v>1172</v>
       </c>
       <c r="F124" t="n">
-        <v>129301813.65</v>
+        <v>164792680</v>
       </c>
     </row>
     <row r="125">
@@ -3914,10 +3914,10 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1020</v>
+        <v>1212</v>
       </c>
       <c r="F125" t="n">
-        <v>145832121.46</v>
+        <v>171234924.25</v>
       </c>
     </row>
     <row r="126">
@@ -3942,10 +3942,10 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>952.1900000000001</v>
+        <v>1219.12</v>
       </c>
       <c r="F126" t="n">
-        <v>134433105.32</v>
+        <v>174264347.86</v>
       </c>
     </row>
     <row r="127">
@@ -3970,10 +3970,10 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>659</v>
+        <v>771</v>
       </c>
       <c r="F127" t="n">
-        <v>92651699.62</v>
+        <v>108629717.98</v>
       </c>
     </row>
     <row r="128">
@@ -3998,10 +3998,10 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>641.4299999999999</v>
+        <v>806.77</v>
       </c>
       <c r="F128" t="n">
-        <v>89870873.40000001</v>
+        <v>112468632.24</v>
       </c>
     </row>
     <row r="129">
@@ -4026,10 +4026,10 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>679.28</v>
+        <v>793.8200000000001</v>
       </c>
       <c r="F129" t="n">
-        <v>96337724.23999999</v>
+        <v>112128019.37</v>
       </c>
     </row>
     <row r="130">
@@ -4054,10 +4054,10 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>589.36</v>
+        <v>719.88</v>
       </c>
       <c r="F130" t="n">
-        <v>83719658.48</v>
+        <v>103213166.37</v>
       </c>
     </row>
     <row r="131">
@@ -4082,10 +4082,10 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>574</v>
+        <v>721</v>
       </c>
       <c r="F131" t="n">
-        <v>81600192.38</v>
+        <v>103060390.19</v>
       </c>
     </row>
     <row r="132">
@@ -4110,10 +4110,10 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>977.8200000000001</v>
+        <v>1143.15</v>
       </c>
       <c r="F132" t="n">
-        <v>138677564.82</v>
+        <v>162718476.32</v>
       </c>
     </row>
     <row r="133">
@@ -4138,10 +4138,10 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>996.99</v>
+        <v>1181.73</v>
       </c>
       <c r="F133" t="n">
-        <v>141073064.56</v>
+        <v>166123399.17</v>
       </c>
     </row>
     <row r="134">
@@ -4166,10 +4166,10 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>932.27</v>
+        <v>1200.2</v>
       </c>
       <c r="F134" t="n">
-        <v>133240466.58</v>
+        <v>168482295.77</v>
       </c>
     </row>
     <row r="135">
@@ -4194,10 +4194,10 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1058.76</v>
+        <v>1242.03</v>
       </c>
       <c r="F135" t="n">
-        <v>151207482.63</v>
+        <v>175189339.97</v>
       </c>
     </row>
     <row r="136">
@@ -4222,10 +4222,10 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>987.1</v>
+        <v>1244.05</v>
       </c>
       <c r="F136" t="n">
-        <v>139472561.22</v>
+        <v>177494150.85</v>
       </c>
     </row>
     <row r="137">
@@ -4250,10 +4250,10 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>679.28</v>
+        <v>773.9</v>
       </c>
       <c r="F137" t="n">
-        <v>95606067.3</v>
+        <v>108930056.98</v>
       </c>
     </row>
     <row r="138">
@@ -4278,10 +4278,10 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>667.66</v>
+        <v>807.54</v>
       </c>
       <c r="F138" t="n">
-        <v>93554946.48999999</v>
+        <v>112719001.38</v>
       </c>
     </row>
     <row r="139">
@@ -4306,10 +4306,10 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>701.39</v>
+        <v>805.5599999999999</v>
       </c>
       <c r="F139" t="n">
-        <v>99752407.33</v>
+        <v>113722030.11</v>
       </c>
     </row>
     <row r="140">
@@ -4334,10 +4334,10 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>623</v>
+        <v>731</v>
       </c>
       <c r="F140" t="n">
-        <v>87955480.73</v>
+        <v>104775228.44</v>
       </c>
     </row>
     <row r="141">
@@ -4362,10 +4362,10 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>606.5700000000001</v>
+        <v>728.09</v>
       </c>
       <c r="F141" t="n">
-        <v>86104142.02</v>
+        <v>104081590.21</v>
       </c>
     </row>
     <row r="142">
@@ -4390,10 +4390,10 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>1016.06</v>
+        <v>1196.79</v>
       </c>
       <c r="F142" t="n">
-        <v>144456221.82</v>
+        <v>170321807.36</v>
       </c>
     </row>
     <row r="143">
@@ -4418,10 +4418,10 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>1032</v>
+        <v>1201</v>
       </c>
       <c r="F143" t="n">
-        <v>145988447.19</v>
+        <v>169561311</v>
       </c>
     </row>
     <row r="144">
@@ -4446,10 +4446,10 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>977.1799999999999</v>
+        <v>1252.98</v>
       </c>
       <c r="F144" t="n">
-        <v>139748815.99</v>
+        <v>176419244.88</v>
       </c>
     </row>
     <row r="145">
@@ -4474,10 +4474,10 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>1114.09</v>
+        <v>1267.86</v>
       </c>
       <c r="F145" t="n">
-        <v>158876006.11</v>
+        <v>178548922.9</v>
       </c>
     </row>
     <row r="146">
@@ -4502,10 +4502,10 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>1053.43</v>
+        <v>1302.42</v>
       </c>
       <c r="F146" t="n">
-        <v>149014190.34</v>
+        <v>185459659.56</v>
       </c>
     </row>
     <row r="147">
@@ -4530,10 +4530,10 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>693.45</v>
+        <v>798.61</v>
       </c>
       <c r="F147" t="n">
-        <v>97974643.34</v>
+        <v>112467107.82</v>
       </c>
     </row>
     <row r="148">
@@ -4558,10 +4558,10 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>713.71</v>
+        <v>851.8099999999999</v>
       </c>
       <c r="F148" t="n">
-        <v>100254610.44</v>
+        <v>118768580.92</v>
       </c>
     </row>
     <row r="149">
@@ -4586,10 +4586,10 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>756.05</v>
+        <v>848.79</v>
       </c>
       <c r="F149" t="n">
-        <v>107441809.69</v>
+        <v>119247509.26</v>
       </c>
     </row>
     <row r="150">
@@ -4614,10 +4614,10 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>649.4</v>
+        <v>758.96</v>
       </c>
       <c r="F150" t="n">
-        <v>91784759.45</v>
+        <v>108883814.93</v>
       </c>
     </row>
     <row r="151">
@@ -4642,10 +4642,10 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>631.9400000000001</v>
+        <v>757.9400000000001</v>
       </c>
       <c r="F151" t="n">
-        <v>89756614.87</v>
+        <v>108429450.39</v>
       </c>
     </row>
     <row r="152">
@@ -4670,10 +4670,10 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>1047</v>
+        <v>1221</v>
       </c>
       <c r="F152" t="n">
-        <v>148623142</v>
+        <v>174109869.88</v>
       </c>
     </row>
     <row r="153">
@@ -4698,10 +4698,10 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>1047.81</v>
+        <v>1213.15</v>
       </c>
       <c r="F153" t="n">
-        <v>148070250.61</v>
+        <v>170841682.47</v>
       </c>
     </row>
     <row r="154">
@@ -4726,10 +4726,10 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>1037.3</v>
+        <v>1277.22</v>
       </c>
       <c r="F154" t="n">
-        <v>148458781.72</v>
+        <v>179579429.41</v>
       </c>
     </row>
     <row r="155">
@@ -4754,10 +4754,10 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>1151.21</v>
+        <v>1294.35</v>
       </c>
       <c r="F155" t="n">
-        <v>164204660.59</v>
+        <v>182114133.41</v>
       </c>
     </row>
     <row r="156">
@@ -4782,10 +4782,10 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>1110.44</v>
+        <v>1286.14</v>
       </c>
       <c r="F156" t="n">
-        <v>156853309.45</v>
+        <v>182907268.08</v>
       </c>
     </row>
     <row r="157">
@@ -4810,10 +4810,10 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>741.9400000000001</v>
+        <v>807.46</v>
       </c>
       <c r="F157" t="n">
-        <v>104591576.56</v>
+        <v>113059345.88</v>
       </c>
     </row>
     <row r="158">
@@ -4838,10 +4838,10 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>720.88</v>
+        <v>855.42</v>
       </c>
       <c r="F158" t="n">
-        <v>101153324.11</v>
+        <v>119154590.15</v>
       </c>
     </row>
     <row r="159">
@@ -4866,10 +4866,10 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>781.12</v>
+        <v>865.46</v>
       </c>
       <c r="F159" t="n">
-        <v>111073860.78</v>
+        <v>121450292.06</v>
       </c>
     </row>
     <row r="160">
@@ -4894,10 +4894,10 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>684.52</v>
+        <v>761.9</v>
       </c>
       <c r="F160" t="n">
-        <v>96714358.48999999</v>
+        <v>109428576.73</v>
       </c>
     </row>
     <row r="161">
@@ -4922,10 +4922,10 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>671.37</v>
+        <v>772.1799999999999</v>
       </c>
       <c r="F161" t="n">
-        <v>95472977.56999999</v>
+        <v>110556045.7</v>
       </c>
     </row>
     <row r="162">
@@ -4950,10 +4950,10 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>1101.81</v>
+        <v>1273.19</v>
       </c>
       <c r="F162" t="n">
-        <v>156926069.72</v>
+        <v>181420836.96</v>
       </c>
     </row>
     <row r="163">
@@ -4978,10 +4978,10 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>1085.34</v>
+        <v>1242.97</v>
       </c>
       <c r="F163" t="n">
-        <v>153674303</v>
+        <v>175161751.86</v>
       </c>
     </row>
     <row r="164">
@@ -5006,10 +5006,10 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>1049.8</v>
+        <v>1292.83</v>
       </c>
       <c r="F164" t="n">
-        <v>150819436.06</v>
+        <v>181739521.29</v>
       </c>
     </row>
     <row r="165">
@@ -5034,10 +5034,10 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>1153.39</v>
+        <v>1270.92</v>
       </c>
       <c r="F165" t="n">
-        <v>164798948.78</v>
+        <v>178694924.96</v>
       </c>
     </row>
     <row r="166">
@@ -5062,10 +5062,10 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>1130.95</v>
+        <v>1283.73</v>
       </c>
       <c r="F166" t="n">
-        <v>159707765.36</v>
+        <v>181894757.6</v>
       </c>
     </row>
     <row r="167">
@@ -5090,10 +5090,10 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>762.95</v>
+        <v>814.74</v>
       </c>
       <c r="F167" t="n">
-        <v>107968778.17</v>
+        <v>114323228.9</v>
       </c>
     </row>
     <row r="168">
@@ -5118,10 +5118,10 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>738.1</v>
+        <v>860.12</v>
       </c>
       <c r="F168" t="n">
-        <v>103747417.74</v>
+        <v>119446771.23</v>
       </c>
     </row>
     <row r="169">
@@ -5146,10 +5146,10 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>790.67</v>
+        <v>875.99</v>
       </c>
       <c r="F169" t="n">
-        <v>112593452.46</v>
+        <v>122516554.86</v>
       </c>
     </row>
     <row r="170">
@@ -5174,10 +5174,10 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>707</v>
+        <v>776</v>
       </c>
       <c r="F170" t="n">
-        <v>100007311.2</v>
+        <v>111443602.37</v>
       </c>
     </row>
     <row r="171">
@@ -5202,10 +5202,10 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>679.28</v>
+        <v>769.92</v>
       </c>
       <c r="F171" t="n">
-        <v>96559881.81</v>
+        <v>110562962.63</v>
       </c>
     </row>
     <row r="172">
@@ -5230,10 +5230,10 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>1112.45</v>
+        <v>1243.98</v>
       </c>
       <c r="F172" t="n">
-        <v>158088515.89</v>
+        <v>177018124.1</v>
       </c>
     </row>
     <row r="173">
@@ -5258,10 +5258,10 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>1092</v>
+        <v>1216</v>
       </c>
       <c r="F173" t="n">
-        <v>154707458.11</v>
+        <v>171481697.15</v>
       </c>
     </row>
     <row r="174">
@@ -5286,10 +5286,10 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>1071.43</v>
+        <v>1252.98</v>
       </c>
       <c r="F174" t="n">
-        <v>153346709.92</v>
+        <v>176090449.84</v>
       </c>
     </row>
     <row r="175">
@@ -5314,10 +5314,10 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>1178.57</v>
+        <v>1243.06</v>
       </c>
       <c r="F175" t="n">
-        <v>168571537.42</v>
+        <v>173939653.66</v>
       </c>
     </row>
     <row r="176">
@@ -5342,10 +5342,10 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>1168.35</v>
+        <v>1275.2</v>
       </c>
       <c r="F176" t="n">
-        <v>165062227.02</v>
+        <v>180750209.67</v>
       </c>
     </row>
     <row r="177">
@@ -5370,10 +5370,10 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>778.77</v>
+        <v>803.5700000000001</v>
       </c>
       <c r="F177" t="n">
-        <v>110169926.65</v>
+        <v>112721867.45</v>
       </c>
     </row>
     <row r="178">
@@ -5398,10 +5398,10 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>774.1900000000001</v>
+        <v>844.76</v>
       </c>
       <c r="F178" t="n">
-        <v>108649739.62</v>
+        <v>116960616.57</v>
       </c>
     </row>
     <row r="179">
@@ -5426,10 +5426,10 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>830.65</v>
+        <v>865.9299999999999</v>
       </c>
       <c r="F179" t="n">
-        <v>118167673.76</v>
+        <v>121542032.28</v>
       </c>
     </row>
     <row r="180">
@@ -5454,10 +5454,10 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>719.12</v>
+        <v>756.97</v>
       </c>
       <c r="F180" t="n">
-        <v>101936981.52</v>
+        <v>109143520.05</v>
       </c>
     </row>
     <row r="181">
@@ -5482,10 +5482,10 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>698.41</v>
+        <v>750</v>
       </c>
       <c r="F181" t="n">
-        <v>99098494.09999999</v>
+        <v>107259537.95</v>
       </c>
     </row>
     <row r="182">
@@ -5510,10 +5510,10 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>1094.06</v>
+        <v>1091.09</v>
       </c>
       <c r="F182" t="n">
-        <v>156035162.26</v>
+        <v>154695823.81</v>
       </c>
     </row>
     <row r="183">
@@ -5538,10 +5538,10 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>1100.5</v>
+        <v>1121.61</v>
       </c>
       <c r="F183" t="n">
-        <v>155981845.11</v>
+        <v>157931626.27</v>
       </c>
     </row>
     <row r="184">
@@ -5566,10 +5566,10 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>1069.65</v>
+        <v>1148.26</v>
       </c>
       <c r="F184" t="n">
-        <v>153193269.63</v>
+        <v>161158100.31</v>
       </c>
     </row>
     <row r="185">
@@ -5594,10 +5594,10 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>1224.24</v>
+        <v>1234.34</v>
       </c>
       <c r="F185" t="n">
-        <v>175101053.4</v>
+        <v>173445583.05</v>
       </c>
     </row>
     <row r="186">
@@ -5622,10 +5622,10 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>1158.21</v>
+        <v>1216.92</v>
       </c>
       <c r="F186" t="n">
-        <v>163785235.8</v>
+        <v>172135282.67</v>
       </c>
     </row>
     <row r="187">
@@ -5650,10 +5650,10 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>832.98</v>
+        <v>824.47</v>
       </c>
       <c r="F187" t="n">
-        <v>117942338.21</v>
+        <v>115422075.95</v>
       </c>
     </row>
     <row r="188">
@@ -5678,10 +5678,10 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>851.0599999999999</v>
+        <v>876.6</v>
       </c>
       <c r="F188" t="n">
-        <v>119366110.79</v>
+        <v>120996060.65</v>
       </c>
     </row>
     <row r="189">
@@ -5706,10 +5706,10 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>902.13</v>
+        <v>895.74</v>
       </c>
       <c r="F189" t="n">
-        <v>128252599.79</v>
+        <v>125346031.84</v>
       </c>
     </row>
     <row r="190">
@@ -5734,10 +5734,10 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>724.38</v>
+        <v>728.36</v>
       </c>
       <c r="F190" t="n">
-        <v>103090132.25</v>
+        <v>104864683.45</v>
       </c>
     </row>
     <row r="191">
@@ -5762,10 +5762,10 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>708.54</v>
+        <v>732.66</v>
       </c>
       <c r="F191" t="n">
-        <v>100386330.88</v>
+        <v>104481983.09</v>
       </c>
     </row>
     <row r="192">
@@ -5790,10 +5790,10 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>1102.09</v>
+        <v>1091.08</v>
       </c>
       <c r="F192" t="n">
-        <v>158109303.53</v>
+        <v>155404880.34</v>
       </c>
     </row>
     <row r="193">
@@ -5818,10 +5818,10 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>1092.73</v>
+        <v>1090.74</v>
       </c>
       <c r="F193" t="n">
-        <v>155750067.54</v>
+        <v>154387115.85</v>
       </c>
     </row>
     <row r="194">
@@ -5846,10 +5846,10 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>1084.71</v>
+        <v>1142.23</v>
       </c>
       <c r="F194" t="n">
-        <v>156096637.21</v>
+        <v>161065522.73</v>
       </c>
     </row>
     <row r="195">
@@ -5874,10 +5874,10 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>1214.88</v>
+        <v>1208.82</v>
       </c>
       <c r="F195" t="n">
-        <v>174900958.05</v>
+        <v>171069297.62</v>
       </c>
     </row>
     <row r="196">
@@ -5902,10 +5902,10 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>1165.8</v>
+        <v>1187.91</v>
       </c>
       <c r="F196" t="n">
-        <v>165567762.41</v>
+        <v>169203081.69</v>
       </c>
     </row>
     <row r="197">
@@ -5930,10 +5930,10 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>796.13</v>
+        <v>759.8</v>
       </c>
       <c r="F197" t="n">
-        <v>113389068.03</v>
+        <v>107376736.45</v>
       </c>
     </row>
     <row r="198">
@@ -5958,10 +5958,10 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>800.98</v>
+        <v>811.03</v>
       </c>
       <c r="F198" t="n">
-        <v>113141833.39</v>
+        <v>112544860.56</v>
       </c>
     </row>
     <row r="199">
@@ -5986,10 +5986,10 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>850.23</v>
+        <v>832.14</v>
       </c>
       <c r="F199" t="n">
-        <v>121632808.35</v>
+        <v>117433800.81</v>
       </c>
     </row>
     <row r="200">
@@ -6014,10 +6014,10 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>735.51</v>
+        <v>718.29</v>
       </c>
       <c r="F200" t="n">
-        <v>105178326.1</v>
+        <v>104322952.01</v>
       </c>
     </row>
     <row r="201">
@@ -6042,10 +6042,10 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>712.38</v>
+        <v>713.39</v>
       </c>
       <c r="F201" t="n">
-        <v>101502813.19</v>
+        <v>102522677.59</v>
       </c>
     </row>
     <row r="202">
@@ -6070,10 +6070,10 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>1117.75</v>
+        <v>1106.59</v>
       </c>
       <c r="F202" t="n">
-        <v>161534498.33</v>
+        <v>158771487.98</v>
       </c>
     </row>
     <row r="203">
@@ -6098,10 +6098,10 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>1108.23</v>
+        <v>1106.21</v>
       </c>
       <c r="F203" t="n">
-        <v>159119081.43</v>
+        <v>157726647.88</v>
       </c>
     </row>
     <row r="204">
@@ -6126,10 +6126,10 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>1078.37</v>
+        <v>1135.55</v>
       </c>
       <c r="F204" t="n">
-        <v>156324065.34</v>
+        <v>161300190.38</v>
       </c>
     </row>
     <row r="205">
@@ -6154,10 +6154,10 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>1207.77</v>
+        <v>1201.75</v>
       </c>
       <c r="F205" t="n">
-        <v>175155783.52</v>
+        <v>171318540.47</v>
       </c>
     </row>
     <row r="206">
@@ -6182,10 +6182,10 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>1182.4</v>
+        <v>1204.83</v>
       </c>
       <c r="F206" t="n">
-        <v>169159968.11</v>
+        <v>172874160.31</v>
       </c>
     </row>
     <row r="207">
@@ -6210,10 +6210,10 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>791.47</v>
+        <v>755.36</v>
       </c>
       <c r="F207" t="n">
-        <v>113554272.51</v>
+        <v>107533181.14</v>
       </c>
     </row>
     <row r="208">
@@ -6238,10 +6238,10 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>812.39</v>
+        <v>822.58</v>
       </c>
       <c r="F208" t="n">
-        <v>115596591.08</v>
+        <v>114986666.16</v>
       </c>
     </row>
     <row r="209">
@@ -6266,10 +6266,10 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>862.34</v>
+        <v>843.99</v>
       </c>
       <c r="F209" t="n">
-        <v>124271788.67</v>
+        <v>119981678.25</v>
       </c>
     </row>
     <row r="210">
@@ -6294,10 +6294,10 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>731.1799999999999</v>
+        <v>714.05</v>
       </c>
       <c r="F210" t="n">
-        <v>105326511.78</v>
+        <v>104469932.55</v>
       </c>
     </row>
     <row r="211">
@@ -6322,10 +6322,10 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>708.21</v>
+        <v>709.21</v>
       </c>
       <c r="F211" t="n">
-        <v>101650699.75</v>
+        <v>102672050.06</v>
       </c>
     </row>
     <row r="212">
@@ -6350,10 +6350,10 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>1120.14</v>
+        <v>1108.95</v>
       </c>
       <c r="F212" t="n">
-        <v>163073370.15</v>
+        <v>160284037.74</v>
       </c>
     </row>
     <row r="213">
@@ -6378,10 +6378,10 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>1110.61</v>
+        <v>1108.59</v>
       </c>
       <c r="F213" t="n">
-        <v>160637512.78</v>
+        <v>159231791.6</v>
       </c>
     </row>
     <row r="214">
@@ -6406,10 +6406,10 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>1102.51</v>
+        <v>1160.97</v>
       </c>
       <c r="F214" t="n">
-        <v>161002686.08</v>
+        <v>166127741.49</v>
       </c>
     </row>
     <row r="215">
@@ -6434,10 +6434,10 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>1234.81</v>
+        <v>1228.66</v>
       </c>
       <c r="F215" t="n">
-        <v>180398018.48</v>
+        <v>176445930.64</v>
       </c>
     </row>
     <row r="216">
@@ -6462,10 +6462,10 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>1184.91</v>
+        <v>1207.38</v>
       </c>
       <c r="F216" t="n">
-        <v>170768730.26</v>
+        <v>174518245.55</v>
       </c>
     </row>
     <row r="217">
@@ -6490,10 +6490,10 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>809.1900000000001</v>
+        <v>772.27</v>
       </c>
       <c r="F217" t="n">
-        <v>116952836.72</v>
+        <v>110751540.19</v>
       </c>
     </row>
     <row r="218">
@@ -6518,10 +6518,10 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>814.11</v>
+        <v>824.33</v>
       </c>
       <c r="F218" t="n">
-        <v>116695949.41</v>
+        <v>116080223.92</v>
       </c>
     </row>
     <row r="219">
@@ -6546,10 +6546,10 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>864.16</v>
+        <v>845.78</v>
       </c>
       <c r="F219" t="n">
-        <v>125453650.74</v>
+        <v>121122740.08</v>
       </c>
     </row>
     <row r="220">
@@ -6574,10 +6574,10 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>732.76</v>
+        <v>715.6</v>
       </c>
       <c r="F220" t="n">
-        <v>106333302.65</v>
+        <v>105468535.58</v>
       </c>
     </row>
     <row r="221">
@@ -6602,10 +6602,10 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>724.0700000000001</v>
+        <v>725.09</v>
       </c>
       <c r="F221" t="n">
-        <v>104693002.1</v>
+        <v>105744920.39</v>
       </c>
     </row>
     <row r="222">
@@ -6630,10 +6630,10 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>1122.58</v>
+        <v>1111.37</v>
       </c>
       <c r="F222" t="n">
-        <v>164638697.33</v>
+        <v>161822590.37</v>
       </c>
     </row>
     <row r="223">
@@ -6658,10 +6658,10 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>1113.05</v>
+        <v>1111.02</v>
       </c>
       <c r="F223" t="n">
-        <v>162182032.66</v>
+        <v>160762795.55</v>
       </c>
     </row>
     <row r="224">
@@ -6686,10 +6686,10 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>1104.88</v>
+        <v>1163.46</v>
       </c>
       <c r="F224" t="n">
-        <v>162542914.52</v>
+        <v>167716998.65</v>
       </c>
     </row>
     <row r="225">
@@ -6714,10 +6714,10 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>1237.46</v>
+        <v>1231.3</v>
       </c>
       <c r="F225" t="n">
-        <v>182123791.91</v>
+        <v>178133896.51</v>
       </c>
     </row>
     <row r="226">
@@ -6742,10 +6742,10 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>1187.47</v>
+        <v>1209.99</v>
       </c>
       <c r="F226" t="n">
-        <v>172405166.01</v>
+        <v>176190612.01</v>
       </c>
     </row>
     <row r="227">
@@ -6770,10 +6770,10 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>810.9299999999999</v>
+        <v>773.9299999999999</v>
       </c>
       <c r="F227" t="n">
-        <v>118071663.3</v>
+        <v>111811042.22</v>
       </c>
     </row>
     <row r="228">
@@ -6798,10 +6798,10 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>815.87</v>
+        <v>826.11</v>
       </c>
       <c r="F228" t="n">
-        <v>117814218.69</v>
+        <v>117192592.85</v>
       </c>
     </row>
     <row r="229">
@@ -6826,10 +6826,10 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>866.04</v>
+        <v>847.61</v>
       </c>
       <c r="F229" t="n">
-        <v>126655842.97</v>
+        <v>122283430.23</v>
       </c>
     </row>
     <row r="230">
@@ -6854,10 +6854,10 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>749.1900000000001</v>
+        <v>731.64</v>
       </c>
       <c r="F230" t="n">
-        <v>109521844.76</v>
+        <v>108631146.53</v>
       </c>
     </row>
     <row r="231">
@@ -6882,10 +6882,10 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>725.62</v>
+        <v>726.65</v>
       </c>
       <c r="F231" t="n">
-        <v>105694545.26</v>
+        <v>106756526.7</v>
       </c>
     </row>
     <row r="232">
@@ -6910,10 +6910,10 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>1125.01</v>
+        <v>1113.77</v>
       </c>
       <c r="F232" t="n">
-        <v>166206424.97</v>
+        <v>163363502.39</v>
       </c>
     </row>
     <row r="233">
@@ -6938,10 +6938,10 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>1137.96</v>
+        <v>1135.88</v>
       </c>
       <c r="F233" t="n">
-        <v>167029932.42</v>
+        <v>165568271.88</v>
       </c>
     </row>
     <row r="234">
@@ -6966,10 +6966,10 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>1107.23</v>
+        <v>1165.94</v>
       </c>
       <c r="F234" t="n">
-        <v>164085455.65</v>
+        <v>169308642.12</v>
       </c>
     </row>
     <row r="235">
@@ -6994,10 +6994,10 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>1240.1</v>
+        <v>1233.92</v>
       </c>
       <c r="F235" t="n">
-        <v>183852156.64</v>
+        <v>179824396.92</v>
       </c>
     </row>
     <row r="236">
@@ -7022,10 +7022,10 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>1190.02</v>
+        <v>1212.59</v>
       </c>
       <c r="F236" t="n">
-        <v>174044085.15</v>
+        <v>177865516.38</v>
       </c>
     </row>
     <row r="237">
@@ -7050,10 +7050,10 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>812.65</v>
+        <v>775.5700000000001</v>
       </c>
       <c r="F237" t="n">
-        <v>119192169.83</v>
+        <v>112872135.11</v>
       </c>
     </row>
     <row r="238">
@@ -7078,10 +7078,10 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>817.62</v>
+        <v>827.88</v>
       </c>
       <c r="F238" t="n">
-        <v>118934185</v>
+        <v>118306649.86</v>
       </c>
     </row>
     <row r="239">
@@ -7106,10 +7106,10 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>867.89</v>
+        <v>849.4299999999999</v>
       </c>
       <c r="F239" t="n">
-        <v>127859859.59</v>
+        <v>123445881.79</v>
       </c>
     </row>
     <row r="240">
@@ -7134,10 +7134,10 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>750.77</v>
+        <v>733.1900000000001</v>
       </c>
       <c r="F240" t="n">
-        <v>110559429.83</v>
+        <v>109660293.33</v>
       </c>
     </row>
     <row r="241">
@@ -7162,10 +7162,10 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>727.17</v>
+        <v>728.2</v>
       </c>
       <c r="F241" t="n">
-        <v>106697592.27</v>
+        <v>107769651.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine workforce attrition and budgets
Co-Authored-By: Chase Dalton <chase.dalton@cognition.ai>
</commit_message>
<xml_diff>
--- a/gdit-workforce-demo/data/finance/fy_headcount_budget.xlsx
+++ b/gdit-workforce-demo/data/finance/fy_headcount_budget.xlsx
@@ -470,10 +470,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>393.57</v>
+        <v>1110</v>
       </c>
       <c r="F2" t="n">
-        <v>55627998.98</v>
+        <v>157101000</v>
       </c>
     </row>
     <row r="3">
@@ -498,10 +498,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>410</v>
+        <v>1145</v>
       </c>
       <c r="F3" t="n">
-        <v>57314975.11</v>
+        <v>160732000</v>
       </c>
     </row>
     <row r="4">
@@ -526,10 +526,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>422.62</v>
+        <v>1180</v>
       </c>
       <c r="F4" t="n">
-        <v>59521264.59</v>
+        <v>166104000</v>
       </c>
     </row>
     <row r="5">
@@ -554,10 +554,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>436.51</v>
+        <v>1215</v>
       </c>
       <c r="F5" t="n">
-        <v>62333830.41</v>
+        <v>170727000</v>
       </c>
     </row>
     <row r="6">
@@ -582,10 +582,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>457.66</v>
+        <v>1175</v>
       </c>
       <c r="F6" t="n">
-        <v>64660473.56</v>
+        <v>166943000</v>
       </c>
     </row>
     <row r="7">
@@ -610,10 +610,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>249.01</v>
+        <v>760</v>
       </c>
       <c r="F7" t="n">
-        <v>35091727.29</v>
+        <v>107011000</v>
       </c>
     </row>
     <row r="8">
@@ -638,10 +638,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>255.04</v>
+        <v>810</v>
       </c>
       <c r="F8" t="n">
-        <v>36126290.57</v>
+        <v>113617000</v>
       </c>
     </row>
     <row r="9">
@@ -666,10 +666,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>287.3</v>
+        <v>795</v>
       </c>
       <c r="F9" t="n">
-        <v>40413394.98</v>
+        <v>112017000</v>
       </c>
     </row>
     <row r="10">
@@ -694,10 +694,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>262.95</v>
+        <v>730</v>
       </c>
       <c r="F10" t="n">
-        <v>37890786.63</v>
+        <v>103567000</v>
       </c>
     </row>
     <row r="11">
@@ -722,10 +722,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>264.88</v>
+        <v>750</v>
       </c>
       <c r="F11" t="n">
-        <v>37981545.76</v>
+        <v>107037000</v>
       </c>
     </row>
     <row r="12">
@@ -750,10 +750,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>450</v>
+        <v>1100</v>
       </c>
       <c r="F12" t="n">
-        <v>63792248.06</v>
+        <v>155378000</v>
       </c>
     </row>
     <row r="13">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>487.05</v>
+        <v>1140</v>
       </c>
       <c r="F13" t="n">
-        <v>68472745.75</v>
+        <v>159697000</v>
       </c>
     </row>
     <row r="14">
@@ -806,10 +806,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>488.91</v>
+        <v>1175</v>
       </c>
       <c r="F14" t="n">
-        <v>69092999.62</v>
+        <v>165299000</v>
       </c>
     </row>
     <row r="15">
@@ -834,10 +834,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>494.96</v>
+        <v>1250</v>
       </c>
       <c r="F15" t="n">
-        <v>70226939.38</v>
+        <v>175663000</v>
       </c>
     </row>
     <row r="16">
@@ -862,10 +862,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>522.09</v>
+        <v>1205</v>
       </c>
       <c r="F16" t="n">
-        <v>73912246.61</v>
+        <v>171017000</v>
       </c>
     </row>
     <row r="17">
@@ -890,10 +890,10 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>304.44</v>
+        <v>745</v>
       </c>
       <c r="F17" t="n">
-        <v>43290447.18</v>
+        <v>105051000</v>
       </c>
     </row>
     <row r="18">
@@ -918,10 +918,10 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>287.15</v>
+        <v>780</v>
       </c>
       <c r="F18" t="n">
-        <v>40283020.43</v>
+        <v>109524000</v>
       </c>
     </row>
     <row r="19">
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>331.33</v>
+        <v>775</v>
       </c>
       <c r="F19" t="n">
-        <v>46389640.68</v>
+        <v>108608000</v>
       </c>
     </row>
     <row r="20">
@@ -974,10 +974,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>296.63</v>
+        <v>705</v>
       </c>
       <c r="F20" t="n">
-        <v>42846572.26</v>
+        <v>99728000</v>
       </c>
     </row>
     <row r="21">
@@ -1002,10 +1002,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>320.56</v>
+        <v>735</v>
       </c>
       <c r="F21" t="n">
-        <v>45999099.81</v>
+        <v>104705000</v>
       </c>
     </row>
     <row r="22">
@@ -1030,10 +1030,10 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>536.85</v>
+        <v>1095</v>
       </c>
       <c r="F22" t="n">
-        <v>76599210.31</v>
+        <v>154523000</v>
       </c>
     </row>
     <row r="23">
@@ -1058,10 +1058,10 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>549.6</v>
+        <v>1150</v>
       </c>
       <c r="F23" t="n">
-        <v>77239188.72</v>
+        <v>161163000</v>
       </c>
     </row>
     <row r="24">
@@ -1086,10 +1086,10 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>592.37</v>
+        <v>1185</v>
       </c>
       <c r="F24" t="n">
-        <v>83839755.43000001</v>
+        <v>167117000</v>
       </c>
     </row>
     <row r="25">
@@ -1114,10 +1114,10 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>600.4</v>
+        <v>1220</v>
       </c>
       <c r="F25" t="n">
-        <v>85449164.59</v>
+        <v>171514000</v>
       </c>
     </row>
     <row r="26">
@@ -1142,10 +1142,10 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>617</v>
+        <v>1185</v>
       </c>
       <c r="F26" t="n">
-        <v>87840102.83</v>
+        <v>168882000</v>
       </c>
     </row>
     <row r="27">
@@ -1170,10 +1170,10 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>366.47</v>
+        <v>755</v>
       </c>
       <c r="F27" t="n">
-        <v>51786570.41</v>
+        <v>106260000</v>
       </c>
     </row>
     <row r="28">
@@ -1198,10 +1198,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>349</v>
+        <v>795</v>
       </c>
       <c r="F28" t="n">
-        <v>48876160.4</v>
+        <v>111628000</v>
       </c>
     </row>
     <row r="29">
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>386</v>
+        <v>765</v>
       </c>
       <c r="F29" t="n">
-        <v>53957910.92</v>
+        <v>107188000</v>
       </c>
     </row>
     <row r="30">
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>363.91</v>
+        <v>735</v>
       </c>
       <c r="F30" t="n">
-        <v>52269502.95</v>
+        <v>104000000</v>
       </c>
     </row>
     <row r="31">
@@ -1282,10 +1282,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>370.48</v>
+        <v>765</v>
       </c>
       <c r="F31" t="n">
-        <v>53147880.87</v>
+        <v>108955000</v>
       </c>
     </row>
     <row r="32">
@@ -1310,10 +1310,10 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>579.37</v>
+        <v>1085</v>
       </c>
       <c r="F32" t="n">
-        <v>82257774.55</v>
+        <v>152959000</v>
       </c>
     </row>
     <row r="33">
@@ -1338,10 +1338,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>617.9400000000001</v>
+        <v>1155</v>
       </c>
       <c r="F33" t="n">
-        <v>86807604.45</v>
+        <v>162181000</v>
       </c>
     </row>
     <row r="34">
@@ -1366,10 +1366,10 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>646</v>
+        <v>1150</v>
       </c>
       <c r="F34" t="n">
-        <v>91085645.68000001</v>
+        <v>161732000</v>
       </c>
     </row>
     <row r="35">
@@ -1394,10 +1394,10 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>654</v>
+        <v>1250</v>
       </c>
       <c r="F35" t="n">
-        <v>92539487.38</v>
+        <v>176130000</v>
       </c>
     </row>
     <row r="36">
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>645.42</v>
+        <v>1225</v>
       </c>
       <c r="F36" t="n">
-        <v>91902063.06999999</v>
+        <v>174621000</v>
       </c>
     </row>
     <row r="37">
@@ -1450,10 +1450,10 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>390</v>
+        <v>750</v>
       </c>
       <c r="F37" t="n">
-        <v>54730504.3</v>
+        <v>105426000</v>
       </c>
     </row>
     <row r="38">
@@ -1478,10 +1478,10 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>391.43</v>
+        <v>800</v>
       </c>
       <c r="F38" t="n">
-        <v>54543549.62</v>
+        <v>112050000</v>
       </c>
     </row>
     <row r="39">
@@ -1506,10 +1506,10 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>415.34</v>
+        <v>755</v>
       </c>
       <c r="F39" t="n">
-        <v>58131340.64</v>
+        <v>106057000</v>
       </c>
     </row>
     <row r="40">
@@ -1534,10 +1534,10 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>398.59</v>
+        <v>725</v>
       </c>
       <c r="F40" t="n">
-        <v>56890360.92</v>
+        <v>102816000</v>
       </c>
     </row>
     <row r="41">
@@ -1562,10 +1562,10 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>409</v>
+        <v>740</v>
       </c>
       <c r="F41" t="n">
-        <v>58901466.55</v>
+        <v>105313000</v>
       </c>
     </row>
     <row r="42">
@@ -1590,10 +1590,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>679</v>
+        <v>1065</v>
       </c>
       <c r="F42" t="n">
-        <v>96291201.8</v>
+        <v>150406000</v>
       </c>
     </row>
     <row r="43">
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>690.24</v>
+        <v>1135</v>
       </c>
       <c r="F43" t="n">
-        <v>96894330</v>
+        <v>159307000</v>
       </c>
     </row>
     <row r="44">
@@ -1646,10 +1646,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>728.83</v>
+        <v>1115</v>
       </c>
       <c r="F44" t="n">
-        <v>103040687.82</v>
+        <v>156568000</v>
       </c>
     </row>
     <row r="45">
@@ -1674,10 +1674,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>730.85</v>
+        <v>1270</v>
       </c>
       <c r="F45" t="n">
-        <v>103704293.05</v>
+        <v>178885000</v>
       </c>
     </row>
     <row r="46">
@@ -1702,10 +1702,10 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>730.92</v>
+        <v>1230</v>
       </c>
       <c r="F46" t="n">
-        <v>104140885.83</v>
+        <v>175118000</v>
       </c>
     </row>
     <row r="47">
@@ -1730,10 +1730,10 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>459.68</v>
+        <v>765</v>
       </c>
       <c r="F47" t="n">
-        <v>64846959.6</v>
+        <v>107494000</v>
       </c>
     </row>
     <row r="48">
@@ -1758,10 +1758,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>465.86</v>
+        <v>800</v>
       </c>
       <c r="F48" t="n">
-        <v>65210258.52</v>
+        <v>111565000</v>
       </c>
     </row>
     <row r="49">
@@ -1786,10 +1786,10 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>493.98</v>
+        <v>780</v>
       </c>
       <c r="F49" t="n">
-        <v>69883696.06999999</v>
+        <v>109522000</v>
       </c>
     </row>
     <row r="50">
@@ -1814,10 +1814,10 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>445.44</v>
+        <v>740</v>
       </c>
       <c r="F50" t="n">
-        <v>63872859.88</v>
+        <v>105026000</v>
       </c>
     </row>
     <row r="51">
@@ -1842,10 +1842,10 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>467.74</v>
+        <v>740</v>
       </c>
       <c r="F51" t="n">
-        <v>67367885.58</v>
+        <v>105118000</v>
       </c>
     </row>
     <row r="52">
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>733.0700000000001</v>
+        <v>1060</v>
       </c>
       <c r="F52" t="n">
-        <v>104107584.23</v>
+        <v>149775000</v>
       </c>
     </row>
     <row r="53">
@@ -1898,10 +1898,10 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>742.0599999999999</v>
+        <v>1140</v>
       </c>
       <c r="F53" t="n">
-        <v>104035098.98</v>
+        <v>159918000</v>
       </c>
     </row>
     <row r="54">
@@ -1926,10 +1926,10 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>775.1</v>
+        <v>1100</v>
       </c>
       <c r="F54" t="n">
-        <v>109403223.34</v>
+        <v>153910000</v>
       </c>
     </row>
     <row r="55">
@@ -1954,10 +1954,10 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>780.12</v>
+        <v>1275</v>
       </c>
       <c r="F55" t="n">
-        <v>110126551.47</v>
+        <v>179989000</v>
       </c>
     </row>
     <row r="56">
@@ -1982,10 +1982,10 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>768</v>
+        <v>1230</v>
       </c>
       <c r="F56" t="n">
-        <v>109708544.74</v>
+        <v>175245000</v>
       </c>
     </row>
     <row r="57">
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>505.02</v>
+        <v>790</v>
       </c>
       <c r="F57" t="n">
-        <v>71351957.33</v>
+        <v>111028000</v>
       </c>
     </row>
     <row r="58">
@@ -2038,10 +2038,10 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>517</v>
+        <v>810</v>
       </c>
       <c r="F58" t="n">
-        <v>72463306.66</v>
+        <v>113011000</v>
       </c>
     </row>
     <row r="59">
@@ -2066,10 +2066,10 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>532</v>
+        <v>785</v>
       </c>
       <c r="F59" t="n">
-        <v>75202714.45999999</v>
+        <v>110602000</v>
       </c>
     </row>
     <row r="60">
@@ -2094,10 +2094,10 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>491.94</v>
+        <v>730</v>
       </c>
       <c r="F60" t="n">
-        <v>70289089.52</v>
+        <v>103302000</v>
       </c>
     </row>
     <row r="61">
@@ -2122,10 +2122,10 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>487.95</v>
+        <v>740</v>
       </c>
       <c r="F61" t="n">
-        <v>70022194.12</v>
+        <v>105290000</v>
       </c>
     </row>
     <row r="62">
@@ -2150,10 +2150,10 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>790.67</v>
+        <v>1070</v>
       </c>
       <c r="F62" t="n">
-        <v>112736279.14</v>
+        <v>151499000</v>
       </c>
     </row>
     <row r="63">
@@ -2178,10 +2178,10 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>840.73</v>
+        <v>1135</v>
       </c>
       <c r="F63" t="n">
-        <v>117641443.76</v>
+        <v>159479000</v>
       </c>
     </row>
     <row r="64">
@@ -2206,10 +2206,10 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>842</v>
+        <v>1095</v>
       </c>
       <c r="F64" t="n">
-        <v>119091743.76</v>
+        <v>153015000</v>
       </c>
     </row>
     <row r="65">
@@ -2234,10 +2234,10 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>860</v>
+        <v>1275</v>
       </c>
       <c r="F65" t="n">
-        <v>121525085.08</v>
+        <v>179822000</v>
       </c>
     </row>
     <row r="66">
@@ -2262,10 +2262,10 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>869.52</v>
+        <v>1240</v>
       </c>
       <c r="F66" t="n">
-        <v>124229413.18</v>
+        <v>176270000</v>
       </c>
     </row>
     <row r="67">
@@ -2290,10 +2290,10 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>551</v>
+        <v>780</v>
       </c>
       <c r="F67" t="n">
-        <v>77940626.09999999</v>
+        <v>109568000</v>
       </c>
     </row>
     <row r="68">
@@ -2318,10 +2318,10 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>567.73</v>
+        <v>795</v>
       </c>
       <c r="F68" t="n">
-        <v>79793390.83</v>
+        <v>110851000</v>
       </c>
     </row>
     <row r="69">
@@ -2346,10 +2346,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>576.6900000000001</v>
+        <v>770</v>
       </c>
       <c r="F69" t="n">
-        <v>81523169.39</v>
+        <v>108418000</v>
       </c>
     </row>
     <row r="70">
@@ -2374,10 +2374,10 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>533.13</v>
+        <v>750</v>
       </c>
       <c r="F70" t="n">
-        <v>76294918.26000001</v>
+        <v>106427000</v>
       </c>
     </row>
     <row r="71">
@@ -2402,10 +2402,10 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>547</v>
+        <v>760</v>
       </c>
       <c r="F71" t="n">
-        <v>78320067.08</v>
+        <v>108246000</v>
       </c>
     </row>
     <row r="72">
@@ -2430,10 +2430,10 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>858.87</v>
+        <v>1065</v>
       </c>
       <c r="F72" t="n">
-        <v>121980038.27</v>
+        <v>150878000</v>
       </c>
     </row>
     <row r="73">
@@ -2458,10 +2458,10 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>892.5700000000001</v>
+        <v>1120</v>
       </c>
       <c r="F73" t="n">
-        <v>125168527.25</v>
+        <v>157587000</v>
       </c>
     </row>
     <row r="74">
@@ -2486,10 +2486,10 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>883.47</v>
+        <v>1095</v>
       </c>
       <c r="F74" t="n">
-        <v>125029963.45</v>
+        <v>153207000</v>
       </c>
     </row>
     <row r="75">
@@ -2514,10 +2514,10 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>911.35</v>
+        <v>1290</v>
       </c>
       <c r="F75" t="n">
-        <v>129066255.41</v>
+        <v>181871000</v>
       </c>
     </row>
     <row r="76">
@@ -2542,10 +2542,10 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>923.61</v>
+        <v>1245</v>
       </c>
       <c r="F76" t="n">
-        <v>132121016.37</v>
+        <v>177280000</v>
       </c>
     </row>
     <row r="77">
@@ -2570,10 +2570,10 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>579.6799999999999</v>
+        <v>770</v>
       </c>
       <c r="F77" t="n">
-        <v>81825841.84999999</v>
+        <v>107940000</v>
       </c>
     </row>
     <row r="78">
@@ -2598,10 +2598,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>607.14</v>
+        <v>785</v>
       </c>
       <c r="F78" t="n">
-        <v>85232695.19</v>
+        <v>109345000</v>
       </c>
     </row>
     <row r="79">
@@ -2626,10 +2626,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>615.08</v>
+        <v>775</v>
       </c>
       <c r="F79" t="n">
-        <v>86608329.64</v>
+        <v>109128000</v>
       </c>
     </row>
     <row r="80">
@@ -2654,10 +2654,10 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>550</v>
+        <v>740</v>
       </c>
       <c r="F80" t="n">
-        <v>78383151.37</v>
+        <v>105078000</v>
       </c>
     </row>
     <row r="81">
@@ -2682,10 +2682,10 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>569.72</v>
+        <v>745</v>
       </c>
       <c r="F81" t="n">
-        <v>81151397.02</v>
+        <v>106165000</v>
       </c>
     </row>
     <row r="82">
@@ -2710,10 +2710,10 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>933.27</v>
+        <v>1070</v>
       </c>
       <c r="F82" t="n">
-        <v>132330832.86</v>
+        <v>151525000</v>
       </c>
     </row>
     <row r="83">
@@ -2738,10 +2738,10 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>955.36</v>
+        <v>1110</v>
       </c>
       <c r="F83" t="n">
-        <v>134272969.14</v>
+        <v>156076000</v>
       </c>
     </row>
     <row r="84">
@@ -2766,10 +2766,10 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>951.8099999999999</v>
+        <v>1095</v>
       </c>
       <c r="F84" t="n">
-        <v>134530701.97</v>
+        <v>153276000</v>
       </c>
     </row>
     <row r="85">
@@ -2794,10 +2794,10 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>1008.03</v>
+        <v>1225</v>
       </c>
       <c r="F85" t="n">
-        <v>143079097.64</v>
+        <v>172742000</v>
       </c>
     </row>
     <row r="86">
@@ -2822,10 +2822,10 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>1001</v>
+        <v>1210</v>
       </c>
       <c r="F86" t="n">
-        <v>143088211.8</v>
+        <v>171619000</v>
       </c>
     </row>
     <row r="87">
@@ -2850,10 +2850,10 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>625.5</v>
+        <v>760</v>
       </c>
       <c r="F87" t="n">
-        <v>88234324.06</v>
+        <v>106522000</v>
       </c>
     </row>
     <row r="88">
@@ -2878,10 +2878,10 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>662</v>
+        <v>775</v>
       </c>
       <c r="F88" t="n">
-        <v>92899159.48</v>
+        <v>107963000</v>
       </c>
     </row>
     <row r="89">
@@ -2906,10 +2906,10 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>669</v>
+        <v>755</v>
       </c>
       <c r="F89" t="n">
-        <v>94062577.95999999</v>
+        <v>106212000</v>
       </c>
     </row>
     <row r="90">
@@ -2934,10 +2934,10 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>592.74</v>
+        <v>750</v>
       </c>
       <c r="F90" t="n">
-        <v>83991091.28</v>
+        <v>106624000</v>
       </c>
     </row>
     <row r="91">
@@ -2962,10 +2962,10 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>607.4299999999999</v>
+        <v>740</v>
       </c>
       <c r="F91" t="n">
-        <v>86756407.31999999</v>
+        <v>105457000</v>
       </c>
     </row>
     <row r="92">
@@ -2990,10 +2990,10 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>978.17</v>
+        <v>1075</v>
       </c>
       <c r="F92" t="n">
-        <v>138800441.08</v>
+        <v>151778000</v>
       </c>
     </row>
     <row r="93">
@@ -3018,10 +3018,10 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>1015.12</v>
+        <v>1100</v>
       </c>
       <c r="F93" t="n">
-        <v>142373739.26</v>
+        <v>154898000</v>
       </c>
     </row>
     <row r="94">
@@ -3046,10 +3046,10 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>1001</v>
+        <v>1095</v>
       </c>
       <c r="F94" t="n">
-        <v>141449526.02</v>
+        <v>153614000</v>
       </c>
     </row>
     <row r="95">
@@ -3074,10 +3074,10 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>1053</v>
+        <v>1245</v>
       </c>
       <c r="F95" t="n">
-        <v>149005565.42</v>
+        <v>174933000</v>
       </c>
     </row>
     <row r="96">
@@ -3102,10 +3102,10 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>1029.88</v>
+        <v>1240</v>
       </c>
       <c r="F96" t="n">
-        <v>146977165.38</v>
+        <v>176126000</v>
       </c>
     </row>
     <row r="97">
@@ -3130,10 +3130,10 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>658</v>
+        <v>755</v>
       </c>
       <c r="F97" t="n">
-        <v>92884140.97</v>
+        <v>105995000</v>
       </c>
     </row>
     <row r="98">
@@ -3158,10 +3158,10 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>694.22</v>
+        <v>775</v>
       </c>
       <c r="F98" t="n">
-        <v>97348220.95999999</v>
+        <v>108024000</v>
       </c>
     </row>
     <row r="99">
@@ -3186,10 +3186,10 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>689.24</v>
+        <v>760</v>
       </c>
       <c r="F99" t="n">
-        <v>96833283.13</v>
+        <v>106981000</v>
       </c>
     </row>
     <row r="100">
@@ -3214,10 +3214,10 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>626.51</v>
+        <v>745</v>
       </c>
       <c r="F100" t="n">
-        <v>89472191.84</v>
+        <v>106000000</v>
       </c>
     </row>
     <row r="101">
@@ -3242,10 +3242,10 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>632</v>
+        <v>745</v>
       </c>
       <c r="F101" t="n">
-        <v>90122755.53</v>
+        <v>106054000</v>
       </c>
     </row>
     <row r="102">
@@ -3270,10 +3270,10 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>1042.34</v>
+        <v>1130</v>
       </c>
       <c r="F102" t="n">
-        <v>148289810.34</v>
+        <v>159881000</v>
       </c>
     </row>
     <row r="103">
@@ -3298,10 +3298,10 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>1064.26</v>
+        <v>1140</v>
       </c>
       <c r="F103" t="n">
-        <v>149868684.22</v>
+        <v>160404000</v>
       </c>
     </row>
     <row r="104">
@@ -3326,10 +3326,10 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>1087.65</v>
+        <v>1150</v>
       </c>
       <c r="F104" t="n">
-        <v>153501822.09</v>
+        <v>161354000</v>
       </c>
     </row>
     <row r="105">
@@ -3354,10 +3354,10 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>1115.54</v>
+        <v>1220</v>
       </c>
       <c r="F105" t="n">
-        <v>157338291.53</v>
+        <v>171278000</v>
       </c>
     </row>
     <row r="106">
@@ -3382,10 +3382,10 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>1110.12</v>
+        <v>1215</v>
       </c>
       <c r="F106" t="n">
-        <v>158297682.96</v>
+        <v>172271000</v>
       </c>
     </row>
     <row r="107">
@@ -3410,10 +3410,10 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>687.25</v>
+        <v>765</v>
       </c>
       <c r="F107" t="n">
-        <v>97213999.81</v>
+        <v>107189000</v>
       </c>
     </row>
     <row r="108">
@@ -3438,10 +3438,10 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>734.13</v>
+        <v>805</v>
       </c>
       <c r="F108" t="n">
-        <v>103113400.21</v>
+        <v>112314000</v>
       </c>
     </row>
     <row r="109">
@@ -3466,10 +3466,10 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>730.16</v>
+        <v>785</v>
       </c>
       <c r="F109" t="n">
-        <v>102775970.44</v>
+        <v>110700000</v>
       </c>
     </row>
     <row r="110">
@@ -3494,10 +3494,10 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>652</v>
+        <v>750</v>
       </c>
       <c r="F110" t="n">
-        <v>92971761.91</v>
+        <v>106751000</v>
       </c>
     </row>
     <row r="111">
@@ -3522,10 +3522,10 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>664.34</v>
+        <v>755</v>
       </c>
       <c r="F111" t="n">
-        <v>94909661.64</v>
+        <v>107294000</v>
       </c>
     </row>
     <row r="112">
@@ -3550,10 +3550,10 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1062.25</v>
+        <v>1075</v>
       </c>
       <c r="F112" t="n">
-        <v>151133689.47</v>
+        <v>152022000</v>
       </c>
     </row>
     <row r="113">
@@ -3578,10 +3578,10 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="F113" t="n">
-        <v>153269447.59</v>
+        <v>153242000</v>
       </c>
     </row>
     <row r="114">
@@ -3606,10 +3606,10 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>1124.01</v>
+        <v>1100</v>
       </c>
       <c r="F114" t="n">
-        <v>158499071.38</v>
+        <v>154361000</v>
       </c>
     </row>
     <row r="115">
@@ -3634,10 +3634,10 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>1154.76</v>
+        <v>1250</v>
       </c>
       <c r="F115" t="n">
-        <v>162636828.87</v>
+        <v>174894000</v>
       </c>
     </row>
     <row r="116">
@@ -3662,10 +3662,10 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>1167.34</v>
+        <v>1255</v>
       </c>
       <c r="F116" t="n">
-        <v>166862638.72</v>
+        <v>178063000</v>
       </c>
     </row>
     <row r="117">
@@ -3690,10 +3690,10 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>712.3</v>
+        <v>760</v>
       </c>
       <c r="F117" t="n">
-        <v>100663600.1</v>
+        <v>106602000</v>
       </c>
     </row>
     <row r="118">
@@ -3718,10 +3718,10 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>777.22</v>
+        <v>795</v>
       </c>
       <c r="F118" t="n">
-        <v>108687131.38</v>
+        <v>110776000</v>
       </c>
     </row>
     <row r="119">
@@ -3746,10 +3746,10 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>762.1</v>
+        <v>795</v>
       </c>
       <c r="F119" t="n">
-        <v>106986316.66</v>
+        <v>112012000</v>
       </c>
     </row>
     <row r="120">
@@ -3774,10 +3774,10 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>676.29</v>
+        <v>735</v>
       </c>
       <c r="F120" t="n">
-        <v>96570630.18000001</v>
+        <v>104657000</v>
       </c>
     </row>
     <row r="121">
@@ -3802,10 +3802,10 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>679.5599999999999</v>
+        <v>735</v>
       </c>
       <c r="F121" t="n">
-        <v>97006889.76000001</v>
+        <v>104628000</v>
       </c>
     </row>
     <row r="122">
@@ -3830,10 +3830,10 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1095.24</v>
+        <v>1120</v>
       </c>
       <c r="F122" t="n">
-        <v>155665695.28</v>
+        <v>157984000</v>
       </c>
     </row>
     <row r="123">
@@ -3858,10 +3858,10 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>1166.33</v>
+        <v>1125</v>
       </c>
       <c r="F123" t="n">
-        <v>163849116.21</v>
+        <v>158253000</v>
       </c>
     </row>
     <row r="124">
@@ -3886,10 +3886,10 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>1172</v>
+        <v>1135</v>
       </c>
       <c r="F124" t="n">
-        <v>164792680</v>
+        <v>159089000</v>
       </c>
     </row>
     <row r="125">
@@ -3914,10 +3914,10 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1212</v>
+        <v>1205</v>
       </c>
       <c r="F125" t="n">
-        <v>171234924.25</v>
+        <v>168367000</v>
       </c>
     </row>
     <row r="126">
@@ -3942,10 +3942,10 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>1219.12</v>
+        <v>1220</v>
       </c>
       <c r="F126" t="n">
-        <v>174264347.86</v>
+        <v>172930000</v>
       </c>
     </row>
     <row r="127">
@@ -3970,10 +3970,10 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>771</v>
+        <v>745</v>
       </c>
       <c r="F127" t="n">
-        <v>108629717.98</v>
+        <v>104680000</v>
       </c>
     </row>
     <row r="128">
@@ -3998,10 +3998,10 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>806.77</v>
+        <v>800</v>
       </c>
       <c r="F128" t="n">
-        <v>112468632.24</v>
+        <v>111426000</v>
       </c>
     </row>
     <row r="129">
@@ -4026,10 +4026,10 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>793.8200000000001</v>
+        <v>790</v>
       </c>
       <c r="F129" t="n">
-        <v>112128019.37</v>
+        <v>111300000</v>
       </c>
     </row>
     <row r="130">
@@ -4054,10 +4054,10 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>719.88</v>
+        <v>740</v>
       </c>
       <c r="F130" t="n">
-        <v>103213166.37</v>
+        <v>105117000</v>
       </c>
     </row>
     <row r="131">
@@ -4082,10 +4082,10 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>721</v>
+        <v>750</v>
       </c>
       <c r="F131" t="n">
-        <v>103060390.19</v>
+        <v>106831000</v>
       </c>
     </row>
     <row r="132">
@@ -4110,10 +4110,10 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>1143.15</v>
+        <v>1140</v>
       </c>
       <c r="F132" t="n">
-        <v>162718476.32</v>
+        <v>161019000</v>
       </c>
     </row>
     <row r="133">
@@ -4138,10 +4138,10 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>1181.73</v>
+        <v>1125</v>
       </c>
       <c r="F133" t="n">
-        <v>166123399.17</v>
+        <v>158480000</v>
       </c>
     </row>
     <row r="134">
@@ -4166,10 +4166,10 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>1200.2</v>
+        <v>1145</v>
       </c>
       <c r="F134" t="n">
-        <v>168482295.77</v>
+        <v>160287000</v>
       </c>
     </row>
     <row r="135">
@@ -4194,10 +4194,10 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1242.03</v>
+        <v>1200</v>
       </c>
       <c r="F135" t="n">
-        <v>175189339.97</v>
+        <v>167288000</v>
       </c>
     </row>
     <row r="136">
@@ -4222,10 +4222,10 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>1244.05</v>
+        <v>1220</v>
       </c>
       <c r="F136" t="n">
-        <v>177494150.85</v>
+        <v>172664000</v>
       </c>
     </row>
     <row r="137">
@@ -4250,10 +4250,10 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>773.9</v>
+        <v>755</v>
       </c>
       <c r="F137" t="n">
-        <v>108930056.98</v>
+        <v>106184000</v>
       </c>
     </row>
     <row r="138">
@@ -4278,10 +4278,10 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>807.54</v>
+        <v>820</v>
       </c>
       <c r="F138" t="n">
-        <v>112719001.38</v>
+        <v>113931000</v>
       </c>
     </row>
     <row r="139">
@@ -4306,10 +4306,10 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>805.5599999999999</v>
+        <v>810</v>
       </c>
       <c r="F139" t="n">
-        <v>113722030.11</v>
+        <v>114324000</v>
       </c>
     </row>
     <row r="140">
@@ -4334,10 +4334,10 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>731</v>
+        <v>745</v>
       </c>
       <c r="F140" t="n">
-        <v>104775228.44</v>
+        <v>106214000</v>
       </c>
     </row>
     <row r="141">
@@ -4362,10 +4362,10 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>728.09</v>
+        <v>750</v>
       </c>
       <c r="F141" t="n">
-        <v>104081590.21</v>
+        <v>106866000</v>
       </c>
     </row>
     <row r="142">
@@ -4390,10 +4390,10 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>1196.79</v>
+        <v>1140</v>
       </c>
       <c r="F142" t="n">
-        <v>170321807.36</v>
+        <v>161075000</v>
       </c>
     </row>
     <row r="143">
@@ -4418,10 +4418,10 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>1201</v>
+        <v>1120</v>
       </c>
       <c r="F143" t="n">
-        <v>169561311</v>
+        <v>158084000</v>
       </c>
     </row>
     <row r="144">
@@ -4446,10 +4446,10 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>1252.98</v>
+        <v>1150</v>
       </c>
       <c r="F144" t="n">
-        <v>176419244.88</v>
+        <v>161197000</v>
       </c>
     </row>
     <row r="145">
@@ -4474,10 +4474,10 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>1267.86</v>
+        <v>1190</v>
       </c>
       <c r="F145" t="n">
-        <v>178548922.9</v>
+        <v>166038000</v>
       </c>
     </row>
     <row r="146">
@@ -4502,10 +4502,10 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>1302.42</v>
+        <v>1210</v>
       </c>
       <c r="F146" t="n">
-        <v>185459659.56</v>
+        <v>171356000</v>
       </c>
     </row>
     <row r="147">
@@ -4530,10 +4530,10 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>798.61</v>
+        <v>750</v>
       </c>
       <c r="F147" t="n">
-        <v>112467107.82</v>
+        <v>105630000</v>
       </c>
     </row>
     <row r="148">
@@ -4558,10 +4558,10 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>851.8099999999999</v>
+        <v>805</v>
       </c>
       <c r="F148" t="n">
-        <v>118768580.92</v>
+        <v>111866000</v>
       </c>
     </row>
     <row r="149">
@@ -4586,10 +4586,10 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>848.79</v>
+        <v>795</v>
       </c>
       <c r="F149" t="n">
-        <v>119247509.26</v>
+        <v>112325000</v>
       </c>
     </row>
     <row r="150">
@@ -4614,10 +4614,10 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>758.96</v>
+        <v>740</v>
       </c>
       <c r="F150" t="n">
-        <v>108883814.93</v>
+        <v>105507000</v>
       </c>
     </row>
     <row r="151">
@@ -4642,10 +4642,10 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>757.9400000000001</v>
+        <v>760</v>
       </c>
       <c r="F151" t="n">
-        <v>108429450.39</v>
+        <v>108413000</v>
       </c>
     </row>
     <row r="152">
@@ -4670,10 +4670,10 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>1221</v>
+        <v>1125</v>
       </c>
       <c r="F152" t="n">
-        <v>174109869.88</v>
+        <v>158683000</v>
       </c>
     </row>
     <row r="153">
@@ -4698,10 +4698,10 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>1213.15</v>
+        <v>1100</v>
       </c>
       <c r="F153" t="n">
-        <v>170841682.47</v>
+        <v>155076000</v>
       </c>
     </row>
     <row r="154">
@@ -4726,10 +4726,10 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>1277.22</v>
+        <v>1135</v>
       </c>
       <c r="F154" t="n">
-        <v>179579429.41</v>
+        <v>158887000</v>
       </c>
     </row>
     <row r="155">
@@ -4754,10 +4754,10 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>1294.35</v>
+        <v>1205</v>
       </c>
       <c r="F155" t="n">
-        <v>182114133.41</v>
+        <v>168253000</v>
       </c>
     </row>
     <row r="156">
@@ -4782,10 +4782,10 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>1286.14</v>
+        <v>1210</v>
       </c>
       <c r="F156" t="n">
-        <v>182907268.08</v>
+        <v>171455000</v>
       </c>
     </row>
     <row r="157">
@@ -4810,10 +4810,10 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>807.46</v>
+        <v>760</v>
       </c>
       <c r="F157" t="n">
-        <v>113059345.88</v>
+        <v>107126000</v>
       </c>
     </row>
     <row r="158">
@@ -4838,10 +4838,10 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>855.42</v>
+        <v>795</v>
       </c>
       <c r="F158" t="n">
-        <v>119154590.15</v>
+        <v>110617000</v>
       </c>
     </row>
     <row r="159">
@@ -4866,10 +4866,10 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>865.46</v>
+        <v>790</v>
       </c>
       <c r="F159" t="n">
-        <v>121450292.06</v>
+        <v>111630000</v>
       </c>
     </row>
     <row r="160">
@@ -4894,10 +4894,10 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>761.9</v>
+        <v>720</v>
       </c>
       <c r="F160" t="n">
-        <v>109428576.73</v>
+        <v>102642000</v>
       </c>
     </row>
     <row r="161">
@@ -4922,10 +4922,10 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>772.1799999999999</v>
+        <v>735</v>
       </c>
       <c r="F161" t="n">
-        <v>110556045.7</v>
+        <v>104697000</v>
       </c>
     </row>
     <row r="162">
@@ -4950,10 +4950,10 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>1273.19</v>
+        <v>1105</v>
       </c>
       <c r="F162" t="n">
-        <v>181420836.96</v>
+        <v>155830000</v>
       </c>
     </row>
     <row r="163">
@@ -4978,10 +4978,10 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>1242.97</v>
+        <v>1105</v>
       </c>
       <c r="F163" t="n">
-        <v>175161751.86</v>
+        <v>155878000</v>
       </c>
     </row>
     <row r="164">
@@ -5006,10 +5006,10 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>1292.83</v>
+        <v>1125</v>
       </c>
       <c r="F164" t="n">
-        <v>181739521.29</v>
+        <v>157548000</v>
       </c>
     </row>
     <row r="165">
@@ -5034,10 +5034,10 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>1270.92</v>
+        <v>1205</v>
       </c>
       <c r="F165" t="n">
-        <v>178694924.96</v>
+        <v>168421000</v>
       </c>
     </row>
     <row r="166">
@@ -5062,10 +5062,10 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>1283.73</v>
+        <v>1240</v>
       </c>
       <c r="F166" t="n">
-        <v>181894757.6</v>
+        <v>175988000</v>
       </c>
     </row>
     <row r="167">
@@ -5090,10 +5090,10 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>814.74</v>
+        <v>775</v>
       </c>
       <c r="F167" t="n">
-        <v>114323228.9</v>
+        <v>109140000</v>
       </c>
     </row>
     <row r="168">
@@ -5118,10 +5118,10 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>860.12</v>
+        <v>800</v>
       </c>
       <c r="F168" t="n">
-        <v>119446771.23</v>
+        <v>111124000</v>
       </c>
     </row>
     <row r="169">
@@ -5146,10 +5146,10 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>875.99</v>
+        <v>800</v>
       </c>
       <c r="F169" t="n">
-        <v>122516554.86</v>
+        <v>113158000</v>
       </c>
     </row>
     <row r="170">
@@ -5174,10 +5174,10 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>776</v>
+        <v>740</v>
       </c>
       <c r="F170" t="n">
-        <v>111443602.37</v>
+        <v>105501000</v>
       </c>
     </row>
     <row r="171">
@@ -5202,10 +5202,10 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>769.92</v>
+        <v>745</v>
       </c>
       <c r="F171" t="n">
-        <v>110562962.63</v>
+        <v>105859000</v>
       </c>
     </row>
     <row r="172">
@@ -5230,10 +5230,10 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>1243.98</v>
+        <v>1140</v>
       </c>
       <c r="F172" t="n">
-        <v>177018124.1</v>
+        <v>160307000</v>
       </c>
     </row>
     <row r="173">
@@ -5258,10 +5258,10 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>1216</v>
+        <v>1120</v>
       </c>
       <c r="F173" t="n">
-        <v>171481697.15</v>
+        <v>157827000</v>
       </c>
     </row>
     <row r="174">
@@ -5286,10 +5286,10 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>1252.98</v>
+        <v>1160</v>
       </c>
       <c r="F174" t="n">
-        <v>176090449.84</v>
+        <v>162298000</v>
       </c>
     </row>
     <row r="175">
@@ -5314,10 +5314,10 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>1243.06</v>
+        <v>1195</v>
       </c>
       <c r="F175" t="n">
-        <v>173939653.66</v>
+        <v>167225000</v>
       </c>
     </row>
     <row r="176">
@@ -5342,10 +5342,10 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>1275.2</v>
+        <v>1215</v>
       </c>
       <c r="F176" t="n">
-        <v>180750209.67</v>
+        <v>172199000</v>
       </c>
     </row>
     <row r="177">
@@ -5370,10 +5370,10 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>803.5700000000001</v>
+        <v>770</v>
       </c>
       <c r="F177" t="n">
-        <v>112721867.45</v>
+        <v>108284000</v>
       </c>
     </row>
     <row r="178">
@@ -5398,10 +5398,10 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>844.76</v>
+        <v>795</v>
       </c>
       <c r="F178" t="n">
-        <v>116960616.57</v>
+        <v>110489000</v>
       </c>
     </row>
     <row r="179">
@@ -5426,10 +5426,10 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>865.9299999999999</v>
+        <v>780</v>
       </c>
       <c r="F179" t="n">
-        <v>121542032.28</v>
+        <v>110792000</v>
       </c>
     </row>
     <row r="180">
@@ -5454,10 +5454,10 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>756.97</v>
+        <v>705</v>
       </c>
       <c r="F180" t="n">
-        <v>109143520.05</v>
+        <v>100729000</v>
       </c>
     </row>
     <row r="181">
@@ -5482,10 +5482,10 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>750</v>
+        <v>730</v>
       </c>
       <c r="F181" t="n">
-        <v>107259537.95</v>
+        <v>103317000</v>
       </c>
     </row>
     <row r="182">
@@ -5510,10 +5510,10 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>1091.09</v>
+        <v>1070</v>
       </c>
       <c r="F182" t="n">
-        <v>154695823.81</v>
+        <v>150262000</v>
       </c>
     </row>
     <row r="183">
@@ -5538,10 +5538,10 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>1121.61</v>
+        <v>1075</v>
       </c>
       <c r="F183" t="n">
-        <v>157931626.27</v>
+        <v>151197000</v>
       </c>
     </row>
     <row r="184">
@@ -5566,10 +5566,10 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>1148.26</v>
+        <v>1095</v>
       </c>
       <c r="F184" t="n">
-        <v>161158100.31</v>
+        <v>153170000</v>
       </c>
     </row>
     <row r="185">
@@ -5594,10 +5594,10 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>1234.34</v>
+        <v>1245</v>
       </c>
       <c r="F185" t="n">
-        <v>173445583.05</v>
+        <v>175054000</v>
       </c>
     </row>
     <row r="186">
@@ -5622,10 +5622,10 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>1216.92</v>
+        <v>1255</v>
       </c>
       <c r="F186" t="n">
-        <v>172135282.67</v>
+        <v>177888000</v>
       </c>
     </row>
     <row r="187">
@@ -5650,10 +5650,10 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>824.47</v>
+        <v>845</v>
       </c>
       <c r="F187" t="n">
-        <v>115422075.95</v>
+        <v>118892000</v>
       </c>
     </row>
     <row r="188">
@@ -5678,10 +5678,10 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>876.6</v>
+        <v>860</v>
       </c>
       <c r="F188" t="n">
-        <v>120996060.65</v>
+        <v>119251000</v>
       </c>
     </row>
     <row r="189">
@@ -5706,10 +5706,10 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>895.74</v>
+        <v>860</v>
       </c>
       <c r="F189" t="n">
-        <v>125346031.84</v>
+        <v>121900000</v>
       </c>
     </row>
     <row r="190">
@@ -5734,10 +5734,10 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>728.36</v>
+        <v>710</v>
       </c>
       <c r="F190" t="n">
-        <v>104864683.45</v>
+        <v>101278000</v>
       </c>
     </row>
     <row r="191">
@@ -5762,10 +5762,10 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>732.66</v>
+        <v>740</v>
       </c>
       <c r="F191" t="n">
-        <v>104481983.09</v>
+        <v>104539000</v>
       </c>
     </row>
     <row r="192">
@@ -5790,10 +5790,10 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>1091.08</v>
+        <v>1110</v>
       </c>
       <c r="F192" t="n">
-        <v>155404880.34</v>
+        <v>156769000</v>
       </c>
     </row>
     <row r="193">
@@ -5818,10 +5818,10 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>1090.74</v>
+        <v>1110</v>
       </c>
       <c r="F193" t="n">
-        <v>154387115.85</v>
+        <v>157261000</v>
       </c>
     </row>
     <row r="194">
@@ -5846,10 +5846,10 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>1142.23</v>
+        <v>1130</v>
       </c>
       <c r="F194" t="n">
-        <v>161065522.73</v>
+        <v>159275000</v>
       </c>
     </row>
     <row r="195">
@@ -5874,10 +5874,10 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>1208.82</v>
+        <v>1245</v>
       </c>
       <c r="F195" t="n">
-        <v>171069297.62</v>
+        <v>176089000</v>
       </c>
     </row>
     <row r="196">
@@ -5902,10 +5902,10 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>1187.91</v>
+        <v>1260</v>
       </c>
       <c r="F196" t="n">
-        <v>169203081.69</v>
+        <v>179626000</v>
       </c>
     </row>
     <row r="197">
@@ -5930,10 +5930,10 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>759.8</v>
+        <v>805</v>
       </c>
       <c r="F197" t="n">
-        <v>107376736.45</v>
+        <v>113879000</v>
       </c>
     </row>
     <row r="198">
@@ -5958,10 +5958,10 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>811.03</v>
+        <v>815</v>
       </c>
       <c r="F198" t="n">
-        <v>112544860.56</v>
+        <v>113654000</v>
       </c>
     </row>
     <row r="199">
@@ -5986,10 +5986,10 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>832.14</v>
+        <v>820</v>
       </c>
       <c r="F199" t="n">
-        <v>117433800.81</v>
+        <v>116759000</v>
       </c>
     </row>
     <row r="200">
@@ -6014,10 +6014,10 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>718.29</v>
+        <v>715</v>
       </c>
       <c r="F200" t="n">
-        <v>104322952.01</v>
+        <v>102582000</v>
       </c>
     </row>
     <row r="201">
@@ -6042,10 +6042,10 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>713.39</v>
+        <v>745</v>
       </c>
       <c r="F201" t="n">
-        <v>102522677.59</v>
+        <v>105975000</v>
       </c>
     </row>
     <row r="202">
@@ -6070,10 +6070,10 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>1106.59</v>
+        <v>1105</v>
       </c>
       <c r="F202" t="n">
-        <v>158771487.98</v>
+        <v>157210000</v>
       </c>
     </row>
     <row r="203">
@@ -6098,10 +6098,10 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>1106.21</v>
+        <v>1105</v>
       </c>
       <c r="F203" t="n">
-        <v>157726647.88</v>
+        <v>157703000</v>
       </c>
     </row>
     <row r="204">
@@ -6126,10 +6126,10 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>1135.55</v>
+        <v>1125</v>
       </c>
       <c r="F204" t="n">
-        <v>161300190.38</v>
+        <v>159736000</v>
       </c>
     </row>
     <row r="205">
@@ -6154,10 +6154,10 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>1201.75</v>
+        <v>1220</v>
       </c>
       <c r="F205" t="n">
-        <v>171318540.47</v>
+        <v>173821000</v>
       </c>
     </row>
     <row r="206">
@@ -6182,10 +6182,10 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>1204.83</v>
+        <v>1235</v>
       </c>
       <c r="F206" t="n">
-        <v>172874160.31</v>
+        <v>177356000</v>
       </c>
     </row>
     <row r="207">
@@ -6210,10 +6210,10 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>755.36</v>
+        <v>795</v>
       </c>
       <c r="F207" t="n">
-        <v>107533181.14</v>
+        <v>113291000</v>
       </c>
     </row>
     <row r="208">
@@ -6238,10 +6238,10 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>822.58</v>
+        <v>805</v>
       </c>
       <c r="F208" t="n">
-        <v>114986666.16</v>
+        <v>113085000</v>
       </c>
     </row>
     <row r="209">
@@ -6266,10 +6266,10 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>843.99</v>
+        <v>810</v>
       </c>
       <c r="F209" t="n">
-        <v>119981678.25</v>
+        <v>116183000</v>
       </c>
     </row>
     <row r="210">
@@ -6294,10 +6294,10 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>714.05</v>
+        <v>715</v>
       </c>
       <c r="F210" t="n">
-        <v>104469932.55</v>
+        <v>103336000</v>
       </c>
     </row>
     <row r="211">
@@ -6322,10 +6322,10 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>709.21</v>
+        <v>745</v>
       </c>
       <c r="F211" t="n">
-        <v>102672050.06</v>
+        <v>106754000</v>
       </c>
     </row>
     <row r="212">
@@ -6350,10 +6350,10 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>1108.95</v>
+        <v>1120</v>
       </c>
       <c r="F212" t="n">
-        <v>160284037.74</v>
+        <v>160519000</v>
       </c>
     </row>
     <row r="213">
@@ -6378,10 +6378,10 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>1108.59</v>
+        <v>1120</v>
       </c>
       <c r="F213" t="n">
-        <v>159231791.6</v>
+        <v>161023000</v>
       </c>
     </row>
     <row r="214">
@@ -6406,10 +6406,10 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>1160.97</v>
+        <v>1140</v>
       </c>
       <c r="F214" t="n">
-        <v>166127741.49</v>
+        <v>163059000</v>
       </c>
     </row>
     <row r="215">
@@ -6434,10 +6434,10 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>1228.66</v>
+        <v>1230</v>
       </c>
       <c r="F215" t="n">
-        <v>176445930.64</v>
+        <v>176539000</v>
       </c>
     </row>
     <row r="216">
@@ -6462,10 +6462,10 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>1207.38</v>
+        <v>1245</v>
       </c>
       <c r="F216" t="n">
-        <v>174518245.55</v>
+        <v>180111000</v>
       </c>
     </row>
     <row r="217">
@@ -6490,10 +6490,10 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>772.27</v>
+        <v>800</v>
       </c>
       <c r="F217" t="n">
-        <v>110751540.19</v>
+        <v>114845000</v>
       </c>
     </row>
     <row r="218">
@@ -6518,10 +6518,10 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>824.33</v>
+        <v>810</v>
       </c>
       <c r="F218" t="n">
-        <v>116080223.92</v>
+        <v>114626000</v>
       </c>
     </row>
     <row r="219">
@@ -6546,10 +6546,10 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>845.78</v>
+        <v>815</v>
       </c>
       <c r="F219" t="n">
-        <v>121122740.08</v>
+        <v>117762000</v>
       </c>
     </row>
     <row r="220">
@@ -6574,10 +6574,10 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>715.6</v>
+        <v>715</v>
       </c>
       <c r="F220" t="n">
-        <v>105468535.58</v>
+        <v>104098000</v>
       </c>
     </row>
     <row r="221">
@@ -6602,10 +6602,10 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>725.09</v>
+        <v>750</v>
       </c>
       <c r="F221" t="n">
-        <v>105744920.39</v>
+        <v>108263000</v>
       </c>
     </row>
     <row r="222">
@@ -6630,10 +6630,10 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>1111.37</v>
+        <v>1095</v>
       </c>
       <c r="F222" t="n">
-        <v>161822590.37</v>
+        <v>158097000</v>
       </c>
     </row>
     <row r="223">
@@ -6658,10 +6658,10 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>1111.02</v>
+        <v>1095</v>
       </c>
       <c r="F223" t="n">
-        <v>160762795.55</v>
+        <v>158594000</v>
       </c>
     </row>
     <row r="224">
@@ -6686,10 +6686,10 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>1163.46</v>
+        <v>1115</v>
       </c>
       <c r="F224" t="n">
-        <v>167716998.65</v>
+        <v>160664000</v>
       </c>
     </row>
     <row r="225">
@@ -6714,10 +6714,10 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>1231.3</v>
+        <v>1275</v>
       </c>
       <c r="F225" t="n">
-        <v>178133896.51</v>
+        <v>184352000</v>
       </c>
     </row>
     <row r="226">
@@ -6742,10 +6742,10 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>1209.99</v>
+        <v>1290</v>
       </c>
       <c r="F226" t="n">
-        <v>176190612.01</v>
+        <v>188002000</v>
       </c>
     </row>
     <row r="227">
@@ -6770,10 +6770,10 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>773.9299999999999</v>
+        <v>825</v>
       </c>
       <c r="F227" t="n">
-        <v>111811042.22</v>
+        <v>119310000</v>
       </c>
     </row>
     <row r="228">
@@ -6798,10 +6798,10 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>826.11</v>
+        <v>840</v>
       </c>
       <c r="F228" t="n">
-        <v>117192592.85</v>
+        <v>119752000</v>
       </c>
     </row>
     <row r="229">
@@ -6826,10 +6826,10 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>847.61</v>
+        <v>840</v>
       </c>
       <c r="F229" t="n">
-        <v>122283430.23</v>
+        <v>122273000</v>
       </c>
     </row>
     <row r="230">
@@ -6854,10 +6854,10 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>731.64</v>
+        <v>725</v>
       </c>
       <c r="F230" t="n">
-        <v>108631146.53</v>
+        <v>106335000</v>
       </c>
     </row>
     <row r="231">
@@ -6882,10 +6882,10 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>726.65</v>
+        <v>765</v>
       </c>
       <c r="F231" t="n">
-        <v>106756526.7</v>
+        <v>111245000</v>
       </c>
     </row>
     <row r="232">
@@ -6910,10 +6910,10 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>1113.77</v>
+        <v>1135</v>
       </c>
       <c r="F232" t="n">
-        <v>163363502.39</v>
+        <v>165077000</v>
       </c>
     </row>
     <row r="233">
@@ -6938,10 +6938,10 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>1135.88</v>
+        <v>1135</v>
       </c>
       <c r="F233" t="n">
-        <v>165568271.88</v>
+        <v>165595000</v>
       </c>
     </row>
     <row r="234">
@@ -6966,10 +6966,10 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>1165.94</v>
+        <v>1155</v>
       </c>
       <c r="F234" t="n">
-        <v>169308642.12</v>
+        <v>167651000</v>
       </c>
     </row>
     <row r="235">
@@ -6994,10 +6994,10 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>1233.92</v>
+        <v>1285</v>
       </c>
       <c r="F235" t="n">
-        <v>179824396.92</v>
+        <v>187163000</v>
       </c>
     </row>
     <row r="236">
@@ -7022,10 +7022,10 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>1212.59</v>
+        <v>1305</v>
       </c>
       <c r="F236" t="n">
-        <v>177865516.38</v>
+        <v>191585000</v>
       </c>
     </row>
     <row r="237">
@@ -7050,10 +7050,10 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>775.5700000000001</v>
+        <v>805</v>
       </c>
       <c r="F237" t="n">
-        <v>112872135.11</v>
+        <v>117273000</v>
       </c>
     </row>
     <row r="238">
@@ -7078,10 +7078,10 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>827.88</v>
+        <v>815</v>
       </c>
       <c r="F238" t="n">
-        <v>118306649.86</v>
+        <v>117041000</v>
       </c>
     </row>
     <row r="239">
@@ -7106,10 +7106,10 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>849.4299999999999</v>
+        <v>820</v>
       </c>
       <c r="F239" t="n">
-        <v>123445881.79</v>
+        <v>120239000</v>
       </c>
     </row>
     <row r="240">
@@ -7134,10 +7134,10 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>733.1900000000001</v>
+        <v>725</v>
       </c>
       <c r="F240" t="n">
-        <v>109660293.33</v>
+        <v>107116000</v>
       </c>
     </row>
     <row r="241">
@@ -7162,10 +7162,10 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>728.2</v>
+        <v>755</v>
       </c>
       <c r="F241" t="n">
-        <v>107769651.97</v>
+        <v>110598000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix fiscal quarter label
Co-Authored-By: Chase Dalton <chase.dalton@cognition.ai>
</commit_message>
<xml_diff>
--- a/gdit-workforce-demo/data/finance/fy_headcount_budget.xlsx
+++ b/gdit-workforce-demo/data/finance/fy_headcount_budget.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Headcount Budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headcount Budget" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>